<commit_message>
Resolved concern on beam notch and identified several missing connection rows
</commit_message>
<xml_diff>
--- a/materials/materials-list.xlsx
+++ b/materials/materials-list.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Buy list'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cut list'!$A$1:$I$56</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sheet goods'!$A$1:$F$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hardware'!$A$1:$D$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hardware'!$A$1:$D$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TBD and assumptions'!$A$1:$C$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -4505,7 +4505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D77"/>
+  <dimension ref="A1:D86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -5453,47 +5453,47 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_top -&gt; beam</t>
+          <t>loft_ceiling -&gt; deck_joist[*]</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL, between the slats. The cap is finish stock doing structural work - it is the slats' seat - so it is fixed on its own account, not by the slat screws alone.</t>
+          <t>construction adhesive + #8 x 2 at 8 in o.c. up into each joist's 1-1/2 bottom edge - 3/4 of ply then 1-1/4 into 3-1/2 of joist. Rev AT: the panel had NO connection row of any kind before this.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>slat[*] -&gt; beam_wrap_top</t>
+          <t>loft_ceiling -&gt; rear_ledger</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>1 x #8 x 3 through the cap into the LVL — 3/4 of cap, 2-1/4 into the beam. Rev AG settles what Rev T left open. slat[22] is the one exception - see below.</t>
+          <t>construction adhesive + #8 x 2 at 8 in o.c. into the ledger's bottom edge</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>slat[22] -&gt; beam_wrap_top</t>
+          <t>loft_ceiling -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -5501,19 +5501,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>1 x #8 x 3, OFFSET INBOARD. slat[22] runs x 105.5 to 107 and the LVL ends at 106.25, so only 3/4 of its 1-1/2 width has beam under the cap - the rest is over beam_end_cap, 3/4 ply. A centred screw lands half in ply. Found by the kernel ray cast.</t>
+          <t>construction adhesive + #8 x 2 at 6 in o.c. into the ledger's bottom edge over the whole 50. Rev AT: tighter than the 8 in field spacing because this is the anchored side of the notch tie - see the beam row below.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>ledge_cleat -&gt; wall:bed</t>
+          <t>loft_ceiling -&gt; deck_joist_tail</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -5521,23 +5521,23 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws into every stud — it carries half an 8 wide lid and whatever is set on it, so it is fixed like a ledger, not tacked like trim</t>
+          <t>construction adhesive + 2 x #8 x 2 into the tail's 1-3/4 of bottom edge, the other anchored side of the notch tie (Rev AT)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>ledge_strut[*] -&gt; ledge_cleat</t>
+          <t>loft_ceiling -&gt; beam</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
@@ -5546,18 +5546,18 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>2 x #8 x 2-1/2 toe-driven into the cleat, plus adhesive</t>
+          <t>construction adhesive + #8 x 2 at 6 in o.c. into the beam's bottom edge over x 3 to 27, then 12 in o.c. beyond. Rev AT: this is the SECOND notch restraint, and it acts in the direction the notch would actually fail. A split from the corner at x 3, z 57.25 runs in +x along the grain, and the piece it separates is the beam's bottom 3-1/2 beyond x 3 - whose bottom face is this z 53.75 line. The same sheet is screwed to side_ledger and deck_joist_tail on the other side of x 3, both solidly bearing, so it is a continuous tie holding that piece up against members that cannot move. It is SECONDARY to beam_wrap_face, which is in the plane of the split and works in shear; this works in screw withdrawal from a 1-3/4 landing that is the LVL's LAMINATED EDGE - screws there cross glue lines, so use the stated spacing, do not over-torque, and do not treat this as the primary. Both go on late, so neither is present while the loft is being framed.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>ledge_strut[*] -&gt; ledge_front_rail</t>
+          <t>beam_wrap_face -&gt; beam</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
@@ -5566,34 +5566,34 @@
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>adhesive + 2 pocket screws from inside the well, angled out of the strut into the back of the rail. Pocket, not toe: a toe screw into 3/4 of poplar from behind breaks out the face, and a screw through the rail's face lands in the strut's end grain.</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. in two rows into the LVL - 3/4 of ply then 1-1/4 into 1-3/4 of beam. Rev AT: OVER x 0 TO 27 THIS IS STRUCTURAL, not a finish fixing: tighten to 6 in o.c. in two rows and glue the full contact area. This panel is the notch reinforcement (see beam_tongue) - it straddles the re-entrant corner at x 3, z 57.25 and runs the full length past the shoulder, so it carries across the corner in shear what the LVL would otherwise carry in cross-grain tension. Keep every screw at least 1 in clear of the corner and out of the notch void below z 57.25 at x 0-3. Rev AT: the wrap had no connection row at all before this - its fixing was never specified and never checked.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_strut[*]</t>
+          <t>beam_wrap_face -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4, 2 per strut, countersunk and filled</t>
+          <t>#8 x 2 at 6 in o.c. into the ledger's y-50 end face, over z 53.75-57.25. Rev AT: part of the notch splice - this is what ties the tongue back to the member it bears on. End-grain withdrawal is poor and irrelevant here: the joint works in shear.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_cleat</t>
+          <t>beam_wrap_face -&gt; deck_joist_tail</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -5601,19 +5601,19 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4 at 12 in o.c., countersunk and filled — the lid is fixed, not hinged</t>
+          <t>#8 x 2 at 6 in o.c. into the tail's y-50 end face, over z 53.75-57.25 - the other half of the notch splice, into the joist sistered to the ledger (Rev AT)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>ledge_cleat_rail -&gt; ledge_front_rail</t>
+          <t>beam_wrap_inner -&gt; beam</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
@@ -5626,14 +5626,14 @@
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-1/4 at 12 in o.c. from inside the well, through the cleat into the rail — screwed from the back so nothing shows on the face</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL. Rev AT: finish fixing only - this panel starts at z 58, 3/4 above the notch corner, so it does no structural work and is not part of the splice. It had no connection row either.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>ledge_cleat_rail -&gt; deck_ply</t>
+          <t>beam_wrap_top -&gt; beam</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -5646,18 +5646,18 @@
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #10 x 3-1/2 down through the cleat and the ply into a joist at each of the 9 joists, and #8 x 2 into the ply between them</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL, between the slats. The cap is finish stock doing structural work - it is the slats' seat - so it is fixed on its own account, not by the slat screws alone.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_front_rail</t>
+          <t>slat[*] -&gt; beam_wrap_top</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
@@ -5666,14 +5666,14 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4 at 12 in o.c. into the rail's 3/4 top edge, countersunk and filled. Rev AM: the lid is fixed, never hinged, so this joint is permanent - and with the three struts holding the rail's top on 7.25 it is a flush line the whole 106 1/4, not a joint that has to be pulled closed at assembly.</t>
+          <t>1 x #8 x 3 through the cap into the LVL — 3/4 of cap, 2-1/4 into the beam. Rev AG settles what Rev T left open. slat[22] is the one exception - see below.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>ledge_rail_splice -&gt; ledge_front_rail</t>
+          <t>slat[22] -&gt; beam_wrap_top</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -5681,19 +5681,19 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-1/4 at 6 in o.c. in two rows, from inside the well through the splice into the back of both rail pieces - 1/2 into the rail's 3/4</t>
+          <t>1 x #8 x 3, OFFSET INBOARD. slat[22] runs x 105.5 to 107 and the LVL ends at 106.25, so only 3/4 of its 1-1/2 width has beam under the cap - the rest is over beam_end_cap, 3/4 ply. A centred screw lands half in ply. Found by the kernel ray cast.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_end_cap</t>
+          <t>ledge_cleat -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
@@ -5701,79 +5701,79 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4, 2 off — the 3/4 x 8 of skirt top edge the lid laps at the stair end (Rev AH)</t>
+          <t>2 x 3 in screws into every stud — it carries half an 8 wide lid and whatever is set on it, so it is fixed like a ledger, not tacked like trim</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>screen_top_plate -&gt; slat[*]</t>
+          <t>ledge_strut[*] -&gt; ledge_cleat</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + 1 x #8 x 2-1/2 angled up through the slat into the plate, driven from the loft side, countersunk and filled; 2 x 1-1/2 16ga pins each slat to hold it while the adhesive cures. Rev AS: was UNSPECIFIED. 16ga alone was proposed and is not enough - the structure table calls this screen the GUARD for a 58 deck, and the ceiling note says a 200 lb lean at its top overloads the slat bases. One real screw per slat at each end (the base already has #8 x 3 into the LVL) makes the top a positive connection; the pins are for assembly, not for load.</t>
+          <t>2 x #8 x 2-1/2 toe-driven into the cleat, plus adhesive</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>screen_top_plate -&gt; ceiling</t>
+          <t>ledge_strut[*] -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>into ceiling framing / blocking — joist location not yet measured</t>
+          <t>adhesive + 2 pocket screws from inside the well, angled out of the strut into the back of the rail. Pocket, not toe: a toe screw into 3/4 of poplar from behind breaks out the face, and a screw through the rail's face lands in the strut's end grain.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>lnd_ledger_bedwall -&gt; wall:bed</t>
+          <t>ledge_lid -&gt; ledge_strut[*]</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>3/8 x 4 lags, 2 per stud</t>
+          <t>#8 x 1-1/4, 2 per strut, countersunk and filled</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>stringer_b -&gt; lnd_rim</t>
+          <t>ledge_lid -&gt; ledge_cleat</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
@@ -5781,19 +5781,19 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>3 x 1/4 x 3-1/2 SDS from inside the box through the rim, before the deck goes on</t>
+          <t>#8 x 1-1/4 at 12 in o.c., countersunk and filled — the lid is fixed, not hinged</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; lnd_ledger_rightwall</t>
+          <t>ledge_cleat_rail -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -5806,14 +5806,14 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>plumb cut on the ledger end + 4 x 1/4 x 4-1/2 SDS into right-wall studs</t>
+          <t>construction adhesive + #8 x 1-1/4 at 12 in o.c. from inside the well, through the cleat into the rail — screwed from the back so nothing shows on the face</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_header</t>
+          <t>ledge_cleat_rail -&gt; deck_ply</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
@@ -5821,19 +5821,19 @@
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>4 x 1/4 x 3-1/2 SDS over y 18-27. Rev AE: the stringer is on the framing now, not on 3/4 of ply, so a 3-1/2 buries 2 in the header.</t>
+          <t>construction adhesive + #10 x 3-1/2 down through the cleat and the ply into a joist at each of the 9 joists, and #8 x 2 into the ply between them</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_king_b</t>
+          <t>ledge_lid -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -5841,19 +5841,19 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS</t>
+          <t>#8 x 1-1/4 at 12 in o.c. into the rail's 3/4 top edge, countersunk and filled. Rev AM: the lid is fixed, never hinged, so this joint is permanent - and with the three struts holding the rail's top on 7.25 it is a flush line the whole 106 1/4, not a joint that has to be pulled closed at assembly.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_trimmer_b</t>
+          <t>ledge_rail_splice -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
@@ -5866,14 +5866,14 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS. Rev AE: the stringer crosses the far jamb pack over z 12-24, so it catches the trimmer as well as the king.</t>
+          <t>construction adhesive + #8 x 1-1/4 at 6 in o.c. in two rows, from inside the well through the splice into the back of both rail pieces - 1/2 into the rail's 3/4</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>hw_rake_nailer -&gt; stringer_a</t>
+          <t>ledge_lid -&gt; ledge_end_cap</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -5881,39 +5881,39 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + 6 x 3 in screws toe-driven through the nailer into the stringer's face. Rev AE: the nailer's raked end (1-1/2 x 30 on the slope) dies straight onto stringer A now that the sheathing between them is gone.</t>
+          <t>#8 x 1-1/4, 2 off — the 3/4 x 8 of skirt top edge the lid laps at the stair end (Rev AH)</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>lnd_rim -&gt; hw_header</t>
+          <t>screen_top_plate -&gt; slat[*]</t>
         </is>
       </c>
       <c r="B71" s="3" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>HUC28 concealed-flange hanger, SD10212 screws straight into the header (flanges would foul the side member on an LUS). Rev AE: no 3/4 facing in the path.</t>
+          <t>construction adhesive + 1 x #8 x 2-1/2 angled up through the slat into the plate, driven from the loft side, countersunk and filled; 2 x 1-1/2 16ga pins each slat to hold it while the adhesive cures. Rev AS: was UNSPECIFIED. 16ga alone was proposed and is not enough - the structure table calls this screen the GUARD for a 58 deck, and the ceiling note says a 200 lb lean at its top overloads the slat bases. One real screw per slat at each end (the base already has #8 x 3 into the LVL) makes the top a positive connection; the pins are for assembly, not for load.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>lnd_rim -&gt; lnd_ledger_rightwall</t>
+          <t>screen_top_plate -&gt; ceiling</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
@@ -5921,59 +5921,59 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>HUC28 concealed-flange hanger (an LUS flange would hang past the ledger end)</t>
+          <t>into ceiling framing / blocking — joist location not yet measured</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>lnd_joist[*] -&gt; lnd_ledger_bedwall</t>
+          <t>lnd_ledger_bedwall -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>LUS24</t>
+          <t>3/8 x 4 lags, 2 per stud</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>lnd_joist[*] -&gt; lnd_rim</t>
+          <t>stringer_b -&gt; lnd_rim</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>LUS24 on the rim's back face</t>
+          <t>3 x 1/4 x 3-1/2 SDS from inside the box through the rim, before the deck goes on</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; lnd_rim</t>
+          <t>stringer_c -&gt; lnd_ledger_rightwall</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
@@ -5986,14 +5986,14 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>2 x A35 at the inside corner, installed before the joists</t>
+          <t>plumb cut on the ledger end + 4 x 1/4 x 4-1/2 SDS into right-wall studs</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; lnd_rim</t>
+          <t>stringer_a -&gt; hw_header</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -6006,32 +6006,212 @@
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS toe-screwed from the stringer's outer face; the side member blocks access from inside the box</t>
+          <t>4 x 1/4 x 3-1/2 SDS over y 18-27. Rev AE: the stringer is on the framing now, not on 3/4 of ply, so a 3-1/2 buries 2 in the header.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
+          <t>stringer_a -&gt; hw_king_b</t>
+        </is>
+      </c>
+      <c r="B77" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C77" s="3" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D77" s="3" t="inlineStr">
+        <is>
+          <t>2 x 1/4 x 3-1/2 SDS</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>stringer_a -&gt; hw_trimmer_b</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>2 x 1/4 x 3-1/2 SDS. Rev AE: the stringer crosses the far jamb pack over z 12-24, so it catches the trimmer as well as the king.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="3" t="inlineStr">
+        <is>
+          <t>hw_rake_nailer -&gt; stringer_a</t>
+        </is>
+      </c>
+      <c r="B79" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C79" s="3" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D79" s="3" t="inlineStr">
+        <is>
+          <t>construction adhesive + 6 x 3 in screws toe-driven through the nailer into the stringer's face. Rev AE: the nailer's raked end (1-1/2 x 30 on the slope) dies straight onto stringer A now that the sheathing between them is gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>lnd_rim -&gt; hw_header</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>HUC28 concealed-flange hanger, SD10212 screws straight into the header (flanges would foul the side member on an LUS). Rev AE: no 3/4 facing in the path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>lnd_rim -&gt; lnd_ledger_rightwall</t>
+        </is>
+      </c>
+      <c r="B81" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C81" s="3" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D81" s="3" t="inlineStr">
+        <is>
+          <t>HUC28 concealed-flange hanger (an LUS flange would hang past the ledger end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>lnd_joist[*] -&gt; lnd_ledger_bedwall</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>LUS24</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>lnd_joist[*] -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B83" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C83" s="3" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D83" s="3" t="inlineStr">
+        <is>
+          <t>LUS24 on the rim's back face</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>lnd_side_member -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>2 x A35 at the inside corner, installed before the joists</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
+        <is>
+          <t>stringer_a -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B85" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C85" s="3" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D85" s="3" t="inlineStr">
+        <is>
+          <t>2 x 1/4 x 3-1/2 SDS toe-screwed from the stringer's outer face; the side member blocks access from inside the box</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
           <t>lnd_blocking[*] -&gt; stringer_b</t>
         </is>
       </c>
-      <c r="B77" s="3" t="n">
+      <c r="B86" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C77" s="3" t="inlineStr">
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>face-screw</t>
         </is>
       </c>
-      <c r="D77" s="3" t="inlineStr">
+      <c r="D86" s="2" t="inlineStr">
         <is>
           <t>2 x 3 in screws each end, toe-driven</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D77"/>
+  <autoFilter ref="A1:D86"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6075,7 +6255,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated from dimensions.yaml rev AS</t>
+          <t>Generated from dimensions.yaml rev AT</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -6121,17 +6301,17 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>MEMBER</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The beam notch's 3/4 ply cheek — NOT in this takeoff</t>
+          <t>The beam notch needs no separate ply cheek (Rev AT)</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>beam_tongue's note prescribes it (LVL makers prohibit bottom notches) but it is not a member, so it is in no drawing, no clash check and no takeoff. Roughly 14 x 27 of 3/4 ply on the inboard face. Where it lands (y 47 1/2-48 1/4) the deck ply is already at z 57 1/4-58 — encode it and resolve that first.</t>
+          <t>It is beam_wrap_face, which already spans the corner on the clear outboard face: adhesive + #8 x 2 at 6 in o.c. over x 0-27, into the tongue above z 57 1/4 and into the ledger and joist-tail end faces below it. Nothing extra to buy — but the wrap's fixing over that first 27 in is STRUCTURAL, not finish, and its screws must stay 1 in clear of the corner and out of the notch void below z 57 1/4.</t>
         </is>
       </c>
     </row>
@@ -6207,12 +6387,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>8 connections carry NO fastener key at all</t>
+          <t>10 connections carry NO fastener key at all</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Filter the Hardware tab for 'NO FASTENER KEY'. verify.py only reports a row that literally says UNSPECIFIED, so these eight pass silently: beam and deck_rim onto hw_top_plate_2, hw_header to both trimmers, hw_top_plate_1 to the header and both kings, and all three stringers to the kicker. Most are ordinary nailing, but the kicker is already an open anchorage item. Worth making verify.py WARN on a missing key — it would change the 0 WARN baseline, so it is your call.</t>
+          <t>Filter the Hardware tab for 'NO FASTENER KEY'. verify.py only reports a row that literally says UNSPECIFIED, so these pass silently: beam -&gt; hw_top_plate_2; deck_rim -&gt; hw_top_plate_2; hw_header -&gt; hw_trimmer_a; hw_header -&gt; hw_trimmer_b; hw_top_plate_1 -&gt; hw_header; hw_top_plate_1 -&gt; hw_king_a; hw_top_plate_1 -&gt; hw_king_b; stringer_a -&gt; kicker; stringer_b -&gt; kicker; stringer_c -&gt; kicker. Most are ordinary nailing, but the kicker is already an open anchorage item. Worth making verify.py WARN on a missing key — it would change the 0 WARN baseline, so it is your call. (Counted from the model, not typed: an earlier hand count said 8.)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Revs AV-AX: nest the sheet goods, re-cut the deck and ceiling ply
</commit_message>
<xml_diff>
--- a/materials/materials-list.xlsx
+++ b/materials/materials-list.xlsx
@@ -10,15 +10,17 @@
     <sheet name="Buy list" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Cut list" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Sheet goods" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Hardware" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TBD and assumptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Cut layout" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Hardware" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="TBD and assumptions" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Buy list'!$A$1:$F$12</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cut list'!$A$1:$I$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sheet goods'!$A$1:$F$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Hardware'!$A$1:$D$90</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'TBD and assumptions'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cut layout'!$A$1:$I$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Hardware'!$A$1:$D$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TBD and assumptions'!$A$1:$C$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -658,7 +660,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>44 pieces total</t>
+          <t>49 pieces total</t>
         </is>
       </c>
     </row>
@@ -688,7 +690,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>44 pieces total, longest 107  ·  LONGEST PIECE NEEDS A 10 FT BOARD</t>
+          <t>49 pieces total, longest 107  ·  LONGEST PIECE NEEDS A 10 FT BOARD</t>
         </is>
       </c>
     </row>
@@ -778,14 +780,14 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>3 pieces; indicative shelf packing, see the Sheet goods tab</t>
+          <t>3 pieces nested at 16% of sheet area; 27.04 sq ft offcut  ·  low yield on a single sheet: the longest piece is 47, so a 4 x 4 half sheet covers it if the yard cuts one  ·  see the Cut layout tab and materials/cut-layout.svg</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>ply-3/4</t>
+          <t>ply-3/4 paint-grade</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -799,7 +801,7 @@
         </is>
       </c>
       <c r="D11" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
@@ -808,7 +810,7 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>37 pieces; indicative shelf packing, see the Sheet goods tab</t>
+          <t>37 pieces nested at 64% of sheet area; 102.29 sq ft offcut  ·  see the Cut layout tab and materials/cut-layout.svg</t>
         </is>
       </c>
     </row>
@@ -1799,11 +1801,11 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>deck_blocking[0..7]</t>
+          <t>deck_blocking[0], deck_blocking[1], deck_blocking[2], deck_blocking[3], deck_blocking[4], deck_blocking[5], deck_blocking[6], deck_blocking[7], deck_seam_blocking[0], deck_seam_blocking[1], deck_seam_blocking[2], deck_seam_blocking[3], deck_seam_blocking[4]</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
@@ -2210,7 +2212,7 @@
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>CUT AS 2 PIECES: 53½ + 53½, each 14¾ — joint on x 53 1/2, over deck_joist[4]</t>
+          <t>CUT AS 2 PIECES: 53½×14¾ + 53½×14¾ — joint on x 53 1/2, over deck_joist[4]</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2257,7 @@
       </c>
       <c r="I33" s="3" t="inlineStr">
         <is>
-          <t>CUT AS 2 PIECES: 53½ + 53½, each 3¼ — joint on x 53 1/2, with the face wrap</t>
+          <t>CUT AS 2 PIECES: 53½×3¼ + 53½×3¼ — joint on x 53 1/2, with the face wrap</t>
         </is>
       </c>
     </row>
@@ -2300,7 +2302,7 @@
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>CUT AS 2 PIECES: 53 1/8 + 53 7/8, each 8 — joint on x 53 1/8, over ledge_strut[1]; no splice needed</t>
+          <t>CUT AS 2 PIECES: 53 1/8×8 + 53 7/8×8 — joint on x 53 1/8, over ledge_strut[1]; no splice needed</t>
         </is>
       </c>
     </row>
@@ -2345,7 +2347,7 @@
       </c>
       <c r="I35" s="3" t="inlineStr">
         <is>
-          <t>CUT AS 2 PIECES: 53 1/8 + 53 1/8, each 9¾ — joint on x 53 1/8, the ledge's joint line</t>
+          <t>CUT AS 2 PIECES: 53 1/8×9¾ + 53 1/8×9¾ — joint on x 53 1/8, the ledge's joint line</t>
         </is>
       </c>
     </row>
@@ -2390,7 +2392,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>CUT AS 3 PIECES: 38¼ + 36 + 32, each 48¼ — joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>CUT AS 3 PIECES: 62¼×24 + 62¼×24¼ + 44×48¼ — two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
         </is>
       </c>
     </row>
@@ -2435,7 +2437,7 @@
       </c>
       <c r="I37" s="3" t="inlineStr">
         <is>
-          <t>CUT AS 2 PIECES: 53 1/8 + 53 1/8, each 10¼ — joint on x 53 1/8 = centre of ledge_strut[1], backed by ledge_rail_splice</t>
+          <t>CUT AS 2 PIECES: 53 1/8×10¼ + 53 1/8×10¼ — joint on x 53 1/8 = centre of ledge_strut[1], backed by ledge_rail_splice</t>
         </is>
       </c>
     </row>
@@ -2480,7 +2482,7 @@
       </c>
       <c r="I38" s="2" t="inlineStr">
         <is>
-          <t>CUT AS 3 PIECES: 38¼ + 36 + 27¾, each 50 — joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>CUT AS 3 PIECES: 38¼×50 + 36×50 + 27¾×50 — three pieces, seams on the joist centres at 38 1/4 and 74 1/4 — every ceiling seam is backed by a joist; clear of all downlights</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3500,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>ledge_lid pc2</t>
+          <t>deck_ply pc1</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -3508,12 +3510,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>53 7/8</t>
+          <t>62¼</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>24</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -3523,14 +3525,14 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>joint on x 53 1/8, over ledge_strut[1]; no splice needed</t>
+          <t>two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>hw_sheath_loft_a</t>
+          <t>deck_ply pc2</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
@@ -3540,21 +3542,29 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>53¾</t>
+          <t>62¼</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>4¼</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr"/>
-      <c r="F6" s="2" t="inlineStr"/>
+          <t>24¼</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>hw_sheath_loft_head</t>
+          <t>ledge_lid pc2</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -3564,25 +3574,29 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>53¾</t>
+          <t>53 7/8</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>45¾</t>
-        </is>
-      </c>
-      <c r="E7" s="3" t="inlineStr"/>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>one notched board; the yaml carries it as hw_sheath_loft_head, hw_sheath_loft_b</t>
+          <t>joint on x 53 1/8, over ledge_strut[1]; no splice needed</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_face pc1</t>
+          <t>hw_sheath_loft_a</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
@@ -3592,29 +3606,21 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>53½</t>
+          <t>53¾</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>14¾</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>joint on x 53 1/2, over deck_joist[4]</t>
-        </is>
-      </c>
+          <t>4¼</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_face pc2</t>
+          <t>hw_sheath_loft_head</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -3624,29 +3630,25 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>53½</t>
+          <t>53¾</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>14¾</t>
-        </is>
-      </c>
-      <c r="E9" s="3" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>45¾</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr"/>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>joint on x 53 1/2, over deck_joist[4]</t>
+          <t>one notched board; the yaml carries it as hw_sheath_loft_head, hw_sheath_loft_b</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_top pc1</t>
+          <t>beam_wrap_face pc1</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
@@ -3661,7 +3663,7 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>3¼</t>
+          <t>14¾</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
@@ -3671,14 +3673,14 @@
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>joint on x 53 1/2, with the face wrap</t>
+          <t>joint on x 53 1/2, over deck_joist[4]</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_top pc2</t>
+          <t>beam_wrap_face pc2</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -3693,7 +3695,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>3¼</t>
+          <t>14¾</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -3703,14 +3705,14 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>joint on x 53 1/2, with the face wrap</t>
+          <t>joint on x 53 1/2, over deck_joist[4]</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid pc1</t>
+          <t>beam_wrap_top pc1</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -3720,12 +3722,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>53 1/8</t>
+          <t>53½</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>3¼</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -3735,14 +3737,14 @@
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>joint on x 53 1/8, over ledge_strut[1]; no splice needed</t>
+          <t>joint on x 53 1/2, with the face wrap</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_inner pc1</t>
+          <t>beam_wrap_top pc2</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -3752,12 +3754,12 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>53 1/8</t>
+          <t>53½</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>9¾</t>
+          <t>3¼</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -3767,14 +3769,14 @@
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>joint on x 53 1/8, the ledge's joint line</t>
+          <t>joint on x 53 1/2, with the face wrap</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_inner pc2</t>
+          <t>ledge_lid pc1</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -3789,7 +3791,7 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>9¾</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
@@ -3799,14 +3801,14 @@
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>joint on x 53 1/8, the ledge's joint line</t>
+          <t>joint on x 53 1/8, over ledge_strut[1]; no splice needed</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>ledge_front_rail pc1</t>
+          <t>beam_wrap_inner pc1</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -3821,7 +3823,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>10¼</t>
+          <t>9¾</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
@@ -3831,14 +3833,14 @@
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>joint on x 53 1/8 = centre of ledge_strut[1], backed by ledge_rail_splice</t>
+          <t>joint on x 53 1/8, the ledge's joint line</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>ledge_front_rail pc2</t>
+          <t>beam_wrap_inner pc2</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
@@ -3853,7 +3855,7 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>10¼</t>
+          <t>9¾</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -3863,14 +3865,14 @@
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>joint on x 53 1/8 = centre of ledge_strut[1], backed by ledge_rail_splice</t>
+          <t>joint on x 53 1/8, the ledge's joint line</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling pc1</t>
+          <t>ledge_front_rail pc1</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -3880,12 +3882,12 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>53 1/8</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>38¼</t>
+          <t>10¼</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
@@ -3895,14 +3897,14 @@
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>joint on x 53 1/8 = centre of ledge_strut[1], backed by ledge_rail_splice</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>loft_ceiling pc2</t>
+          <t>ledge_front_rail pc2</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
@@ -3912,12 +3914,12 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>53 1/8</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>36</t>
+          <t>10¼</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -3927,14 +3929,14 @@
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>joint on x 53 1/8 = centre of ledge_strut[1], backed by ledge_rail_splice</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling pc3</t>
+          <t>loft_ceiling pc1</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -3949,7 +3951,7 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>27¾</t>
+          <t>38¼</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr">
@@ -3959,14 +3961,14 @@
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>three pieces, seams on the joist centres at 38 1/4 and 74 1/4 — every ceiling seam is backed by a joist; clear of all downlights</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>hw_sheath_stair</t>
+          <t>loft_ceiling pc2</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
@@ -3981,20 +3983,24 @@
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>44¼</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr"/>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>one notched board; the yaml carries it as hw_sheath_stair, ledge_end_cap, beam_end_cap</t>
+          <t>three pieces, seams on the joist centres at 38 1/4 and 74 1/4 — every ceiling seam is backed by a joist; clear of all downlights</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>deck_ply pc1</t>
+          <t>loft_ceiling pc3</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -4004,12 +4010,12 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>48¼</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>38¼</t>
+          <t>27¾</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
@@ -4019,14 +4025,14 @@
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>three pieces, seams on the joist centres at 38 1/4 and 74 1/4 — every ceiling seam is backed by a joist; clear of all downlights</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>deck_ply pc2</t>
+          <t>hw_sheath_stair</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
@@ -4036,22 +4042,18 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>48¼</t>
+          <t>50</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>36</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
+          <t>44¼</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>one notched board; the yaml carries it as hw_sheath_stair, ledge_end_cap, beam_end_cap</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4075,7 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>32</t>
+          <t>44</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
@@ -4083,7 +4085,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>joints on deck_joist centres x 38 1/4 and 74 1/4</t>
+          <t>two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4589,1644 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D90"/>
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Piece</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>From edge X</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>From edge Y</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Grain</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Flag</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>ply-1/2</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>hw_header#ply-1/2</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>47</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>9¼</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>ply-1/2</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>hw_jamb_ply_a</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>3½</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>9 3/8</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr"/>
+      <c r="I3" s="3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>ply-1/2</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>hw_jamb_ply_b</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>40</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>3½</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>13</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>deck_ply pc2</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>24¼</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>62¼</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ledge_lid pc2</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>53 7/8</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>24 3/8</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>hw_sheath_loft_a</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>4¼</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>53¾</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>32½</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>beam_wrap_top pc1</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>3¼</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>53½</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>36 7/8</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>beam_wrap_top pc2</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>3¼</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>53½</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>40¼</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>ledge_rail_splice</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>7¼</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>36 7/8</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>53 5/8</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>nk_wrap_bedwall</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>41½</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>28¼</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>62 3/8</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr"/>
+      <c r="I11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>deck_ply pc1</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>62¼</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>beam_wrap_face pc1</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>14¾</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>53½</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>24 1/8</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ledge_lid pc1</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>53 1/8</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>nk_soffit_rake</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>37.8</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>28¼</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>62 3/8</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr"/>
+      <c r="I15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>tread[1]</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>9 1/8</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>25½</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>37.93</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>62 3/8</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>hw_sheath_loft_head</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>45¾</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>53¾</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>nk_wrap_shortwall</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>28¼</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>16.3</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>53 7/8</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>nk_soffit_flat</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>28¼</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>14.01</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>70.3</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr"/>
+      <c r="I19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>tread[3]</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>9 1/8</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>25½</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>28 3/8</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>70.3</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>riser[2]</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>8¼</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>25½</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>37 5/8</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>70.3</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>tread[2]</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>25½</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>9 1/8</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>84 7/16</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>beam_wrap_face pc2</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>14¾</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>53½</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>ledge_front_rail pc1</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>10¼</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>53 1/8</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>14 7/8</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>ledge_front_rail pc2</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>10¼</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>53 1/8</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>25¼</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>beam_wrap_inner pc1</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>9¾</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>53 1/8</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>35 5/8</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>lnd_ply</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>27 7/8</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>53 5/8</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr"/>
+      <c r="I27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>tread[4]</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>9 1/8</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>53 5/8</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>tread[5]</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>9 1/8</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>37¼</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>53 5/8</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>riser[3]</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>25½</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>8¼</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>77¾</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>riser[1]</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>25½</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>7½</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G31" s="3" t="inlineStr">
+        <is>
+          <t>86 1/8</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr"/>
+      <c r="I31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>beam_wrap_inner pc2</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>9¾</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>53 1/8</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I32" s="2" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>loft_ceiling pc2</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>36</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>9 7/8</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr"/>
+      <c r="I33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>stringer_a_skin</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>53¼</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>riser[6]</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>8¼</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>24 1/8</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>53¼</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>riser[4]</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="inlineStr">
+        <is>
+          <t>8¼</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>75 3/8</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>riser[5]</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>8¼</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>83¾</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr"/>
+      <c r="I37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>hw_sheath_stair</t>
+        </is>
+      </c>
+      <c r="D38" s="2" t="inlineStr">
+        <is>
+          <t>44¼</t>
+        </is>
+      </c>
+      <c r="E38" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>rotated</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>loft_ceiling pc1</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>38¼</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G39" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr"/>
+      <c r="I39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>loft_ceiling pc3</t>
+        </is>
+      </c>
+      <c r="D40" s="2" t="inlineStr">
+        <is>
+          <t>27¾</t>
+        </is>
+      </c>
+      <c r="E40" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>ply-3/4 paint-grade</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>deck_ply pc3</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>48¼</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="G41" s="3" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr"/>
+      <c r="I41" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I41"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -4855,7 +6494,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>deck_ply -&gt; side_ledger</t>
+          <t>deck_seam_blocking[0] -&gt; deck_joist[0]</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -4863,19 +6502,19 @@
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. — structural, not just an edge fixing, because the ply diaphragm is what keeps the shallow ledger from rolling under the beam's eccentric load</t>
+          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[0] here and deck_joist[1] at the far end, which carries no row of its own</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>deck_ply -&gt; rear_ledger</t>
+          <t>deck_seam_blocking[1] -&gt; deck_joist[1]</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -4883,19 +6522,19 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c., same as the side ledger — Rev AO drops rear_ledger to deck level so the ply runs over its top the same way</t>
+          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[1] here and deck_joist[2] at the far end, which carries no row of its own</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>beam -&gt; hw_top_plate_2</t>
+          <t>deck_seam_blocking[2] -&gt; deck_joist[2]</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
@@ -4903,19 +6542,19 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[2] here and deck_joist[3] at the far end, which carries no row of its own</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>deck_rim -&gt; hw_top_plate_2</t>
+          <t>deck_seam_blocking[3] -&gt; deck_joist[3]</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -4923,19 +6562,19 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[3] here and deck_joist[4] at the far end, which carries no row of its own</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>rear_ledger -&gt; wall:bed</t>
+          <t>deck_seam_blocking[4] -&gt; deck_joist[4]</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -4943,39 +6582,39 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>3/8 x 4 lags, 2 per stud staggered, into every stud - the same fastener as lnd_ledger_bedwall. Rev AS: was the sizeless 'lags into every stud'. 1 1/2 of 2x4 ledger + 5/8 of board = 2 1/8 crossed, 1 7/8 of embedment.</t>
+          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[4] here and deck_joist[5] at the far end, which carries no row of its own</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>side_ledger -&gt; wall:window</t>
+          <t>deck_ply -&gt; deck_seam_blocking[*]</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>1/4 x 4 structural screws, 2 per stud staggered top and bottom, plus a pair within 6 in of y 50 — FIELD, confirm a stud lands there or add blocking in the wall</t>
+          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. through BOTH panel edges - the seam is a butt joint in the deck diaphragm and both sides land on this block (Rev AV)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>hw_header -&gt; hw_trimmer_a</t>
+          <t>deck_ply -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -4988,14 +6627,14 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. — structural, not just an edge fixing, because the ply diaphragm is what keeps the shallow ledger from rolling under the beam's eccentric load</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>hw_header -&gt; hw_trimmer_b</t>
+          <t>deck_ply -&gt; rear_ledger</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -5008,14 +6647,14 @@
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c., same as the side ledger — Rev AO drops rear_ledger to deck level so the ply runs over its top the same way</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>hw_jamb_ply_a -&gt; hw_bottom_plate_a</t>
+          <t>beam -&gt; hw_top_plate_2</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -5028,14 +6667,14 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>bears with the trimmer; held by the pack nailing below</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>hw_jamb_ply_b -&gt; hw_bottom_plate_b</t>
+          <t>deck_rim -&gt; hw_top_plate_2</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -5048,14 +6687,14 @@
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>bears with the trimmer; held by the pack nailing below</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>hw_trimmer_a -&gt; hw_king_a</t>
+          <t>rear_ledger -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
@@ -5063,19 +6702,19 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
+          <t>3/8 x 4 lags, 2 per stud staggered, into every stud - the same fastener as lnd_ledger_bedwall. Rev AS: was the sizeless 'lags into every stud'. 1 1/2 of 2x4 ledger + 5/8 of board = 2 1/8 crossed, 1 7/8 of embedment.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>hw_trimmer_b -&gt; hw_king_b</t>
+          <t>side_ledger -&gt; wall:window</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -5083,19 +6722,19 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
+          <t>1/4 x 4 structural screws, 2 per stud staggered top and bottom, plus a pair within 6 in of y 50 — FIELD, confirm a stud lands there or add blocking in the wall</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>hw_top_plate_2 -&gt; hw_top_plate_1</t>
+          <t>hw_header -&gt; hw_trimmer_a</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
@@ -5108,14 +6747,14 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>16d at 16 in o.c., staggered — the upper plate laps the lower at the wall's ends</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>hw_king_a -&gt; hw_bottom_plate_a</t>
+          <t>hw_header -&gt; hw_trimmer_b</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -5128,14 +6767,14 @@
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>hw_king_b -&gt; hw_bottom_plate_b</t>
+          <t>hw_jamb_ply_a -&gt; hw_bottom_plate_a</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -5148,14 +6787,14 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate. This is the stud the beam's stair-end reaction comes down; Rev AG's connection audit found the post asserted in prose and never declared.</t>
+          <t>bears with the trimmer; held by the pack nailing below</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>hw_top_plate_1 -&gt; hw_header</t>
+          <t>hw_jamb_ply_b -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -5168,14 +6807,14 @@
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>bears with the trimmer; held by the pack nailing below</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>hw_top_plate_1 -&gt; hw_king_a</t>
+          <t>hw_trimmer_a -&gt; hw_king_a</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
@@ -5183,19 +6822,19 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>hw_top_plate_1 -&gt; hw_king_b</t>
+          <t>hw_trimmer_b -&gt; hw_king_b</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -5203,19 +6842,19 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>hw_bottom_plate_a -&gt; floor</t>
+          <t>hw_top_plate_2 -&gt; hw_top_plate_1</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
@@ -5223,19 +6862,19 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>UNSPECIFIED — declared open</t>
+          <t>16d at 16 in o.c., staggered — the upper plate laps the lower at the wall's ends</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>hw_bottom_plate_b -&gt; floor</t>
+          <t>hw_king_a -&gt; hw_bottom_plate_a</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -5243,23 +6882,23 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>UNSPECIFIED — declared open</t>
+          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>nk_bedwall_stud[*] -&gt; hw_bottom_plate_a</t>
+          <t>hw_king_b -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
@@ -5268,18 +6907,18 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven each stud</t>
+          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate. This is the stud the beam's stair-end reaction comes down; Rev AG's connection audit found the post asserted in prose and never declared.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>nk_bedwall_cap -&gt; nk_bedwall_stud[*]</t>
+          <t>hw_top_plate_1 -&gt; hw_header</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
@@ -5288,14 +6927,14 @@
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws through the cap into each stud</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>lnd_ledger_bedwall -&gt; nk_bedwall_cap</t>
+          <t>hw_top_plate_1 -&gt; hw_king_a</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
@@ -5308,14 +6947,14 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>3 in screws up through the cap into the ledger at each stud — secondary only, the ledger's own load path is its lags into the bed-wall studs</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>lnd_ledger_rightwall -&gt; nk_bedwall_cap</t>
+          <t>hw_top_plate_1 -&gt; hw_king_b</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -5328,14 +6967,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>3 in screws up through the cap, at the cap's right-hand end</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; nk_bedwall_cap</t>
+          <t>hw_bottom_plate_a -&gt; floor</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
@@ -5343,79 +6982,79 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws up through the cap into the side member</t>
+          <t>UNSPECIFIED — declared open</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>nk_shortwall_strut[*] -&gt; hw_bottom_plate_b</t>
+          <t>hw_bottom_plate_b -&gt; floor</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven each strut</t>
+          <t>UNSPECIFIED — declared open</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>hw_rake_nailer -&gt; hw_trimmer_b</t>
+          <t>nk_bedwall_stud[*] -&gt; hw_bottom_plate_a</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>3 x 3 in screws through the trimmer into the nailer's end</t>
+          <t>2 x 3 in screws toe-driven each stud</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; hw_header</t>
+          <t>nk_bedwall_cap -&gt; nk_bedwall_stud[*]</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>6 × 1/4 × 4 structural screws. Rev AE: direct into the header, no 3/4 facing in the path, so 4 in reaches the depth 5 in used to.</t>
+          <t>2 x 3 in screws through the cap into each stud</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>lnd_ledger_rightwall -&gt; wall:right</t>
+          <t>lnd_ledger_bedwall -&gt; nk_bedwall_cap</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
@@ -5423,19 +7062,19 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>1/4 x 4 flat-head structural screws (SDWS22400 or equal), 2 per stud staggered. Rev AS: the wall is 5/8 drywall on wood studs, so a screw crosses 1 1/2 of 2x8 ledger + 5/8 of board = 2 1/8 before it reaches the stud; a 4 leaves 1 7/8 of embedment. Do not substitute 3 1/2 here - that is only 1 3/8 in the stud.</t>
+          <t>3 in screws up through the cap into the ledger at each stud — secondary only, the ledger's own load path is its lags into the bed-wall studs</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; wall:right</t>
+          <t>lnd_ledger_rightwall -&gt; nk_bedwall_cap</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -5443,19 +7082,19 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>1/4 x 4 flat-head structural screws, 2 per stud into every stud the stringer crosses. Rev AS: was the bare Rev T phrase 'fastens to the right wall', which specified nothing. Same 2 1/8 of ledger + board to cross as lnd_ledger_rightwall.</t>
+          <t>3 in screws up through the cap, at the cap's right-hand end</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>stringer_a_skin -&gt; stringer_a</t>
+          <t>lnd_side_member -&gt; nk_bedwall_cap</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
@@ -5463,39 +7102,39 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + 1-1/2 x 16ga finish nails at 8 in o.c. into the stringer's outer face (3/4 penetration)</t>
+          <t>2 x 3 in screws up through the cap into the side member</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; stringer_a_skin</t>
+          <t>nk_shortwall_strut[*] -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>1-1/2 x 16ga finish nails at 8 in o.c. through the skin into the cleat, plus adhesive</t>
+          <t>2 x 3 in screws toe-driven each strut</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; hw_bottom_plate_b</t>
+          <t>hw_rake_nailer -&gt; hw_trimmer_b</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
@@ -5508,14 +7147,14 @@
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>2 x #10 x 3 screws through the plate's end into the cleat</t>
+          <t>3 x 3 in screws through the trimmer into the nailer's end</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; stringer_a</t>
+          <t>lnd_side_member -&gt; hw_header</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -5523,19 +7162,19 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>adhesive + 3 x #10 x 2-1/2 screws up through the cleat's ripped top into the stringer, over the 5 in of angled contact at its downhill end</t>
+          <t>6 × 1/4 × 4 structural screws. Rev AE: direct into the header, no 3/4 facing in the path, so 4 in reaches the depth 5 in used to.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; floor</t>
+          <t>lnd_ledger_rightwall -&gt; wall:right</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
@@ -5543,19 +7182,19 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>3 x #10 x 3 screws into the subfloor</t>
+          <t>1/4 x 4 flat-head structural screws (SDWS22400 or equal), 2 per stud staggered. Rev AS: the wall is 5/8 drywall on wood studs, so a screw crosses 1 1/2 of 2x8 ledger + 5/8 of board = 2 1/8 before it reaches the stud; a 4 leaves 1 7/8 of embedment. Do not substitute 3 1/2 here - that is only 1 3/8 in the stud.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; kicker</t>
+          <t>stringer_c -&gt; wall:right</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -5563,19 +7202,19 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>1/4 x 4 flat-head structural screws, 2 per stud into every stud the stringer crosses. Rev AS: was the bare Rev T phrase 'fastens to the right wall', which specified nothing. Same 2 1/8 of ledger + board to cross as lnd_ledger_rightwall.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>stringer_b -&gt; kicker</t>
+          <t>stringer_a_skin -&gt; stringer_a</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
@@ -5583,19 +7222,19 @@
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>construction adhesive + 1-1/2 x 16ga finish nails at 8 in o.c. into the stringer's outer face (3/4 penetration)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; kicker</t>
+          <t>stringer_a_skin_cleat -&gt; stringer_a_skin</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -5603,23 +7242,23 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>1-1/2 x 16ga finish nails at 8 in o.c. through the skin into the cleat, plus adhesive</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; deck_joist[*]</t>
+          <t>stringer_a_skin_cleat -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C53" s="3" t="inlineStr">
         <is>
@@ -5628,14 +7267,14 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 8 in o.c. up into each joist's 1-1/2 bottom edge - 3/4 of ply then 1-1/4 into 3-1/2 of joist. Rev AT: the panel had NO connection row of any kind before this.</t>
+          <t>2 x #10 x 3 screws through the plate's end into the cleat</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; rear_ledger</t>
+          <t>stringer_a_skin_cleat -&gt; stringer_a</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -5643,19 +7282,19 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 8 in o.c. into the ledger's bottom edge</t>
+          <t>adhesive + 3 x #10 x 2-1/2 screws up through the cleat's ripped top into the stringer, over the 5 in of angled contact at its downhill end</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; side_ledger</t>
+          <t>stringer_a_skin_cleat -&gt; floor</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
@@ -5663,19 +7302,19 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 6 in o.c. into the ledger's bottom edge over the whole 50. Rev AT: tighter than the 8 in field spacing because this is the anchored side of the notch tie - see the beam row below.</t>
+          <t>3 x #10 x 3 screws into the subfloor</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; deck_joist_tail</t>
+          <t>stringer_a -&gt; kicker</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -5683,19 +7322,19 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + 2 x #8 x 2 into the tail's 1-3/4 of bottom edge, the other anchored side of the notch tie (Rev AT)</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; beam</t>
+          <t>stringer_b -&gt; kicker</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
@@ -5703,19 +7342,19 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 6 in o.c. into the beam's bottom edge over x 3 to 27, then 12 in o.c. beyond. Rev AT: this is the SECOND notch restraint, and it acts in the direction the notch would actually fail. A split from the corner at x 3, z 57.25 runs in +x along the grain, and the piece it separates is the beam's bottom 3-1/2 beyond x 3 - whose bottom face is this z 53.75 line. The same sheet is screwed to side_ledger and deck_joist_tail on the other side of x 3, both solidly bearing, so it is a continuous tie holding that piece up against members that cannot move. It is SECONDARY to beam_wrap_face, which is in the plane of the split and works in shear; this works in screw withdrawal from a 1-3/4 landing that is the LVL's LAMINATED EDGE - screws there cross glue lines, so use the stated spacing, do not over-torque, and do not treat this as the primary. Both go on late, so neither is present while the loft is being framed.</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_face -&gt; beam</t>
+          <t>stringer_c -&gt; kicker</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -5723,23 +7362,23 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. in two rows into the LVL - 3/4 of ply then 1-1/4 into 1-3/4 of beam. Rev AT: OVER x 0 TO 27 THIS IS STRUCTURAL, not a finish fixing: tighten to 6 in o.c. in two rows and glue the full contact area. This panel is the notch reinforcement (see beam_tongue) - it straddles the re-entrant corner at x 3, z 57.25 and runs the full length past the shoulder, so it carries across the corner in shear what the LVL would otherwise carry in cross-grain tension. Keep every screw at least 1 in clear of the corner and out of the notch void below z 57.25 at x 0-3. Rev AT: the wrap had no connection row at all before this - its fixing was never specified and never checked.</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_face -&gt; side_ledger</t>
+          <t>loft_ceiling -&gt; deck_joist[*]</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
@@ -5748,14 +7387,14 @@
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>#8 x 2 at 6 in o.c. into the ledger's y-50 end face, over z 53.75-57.25. Rev AT: part of the notch splice - this is what ties the tongue back to the member it bears on. End-grain withdrawal is poor and irrelevant here: the joint works in shear.</t>
+          <t>construction adhesive + #8 x 2 at 8 in o.c. up into each joist's 1-1/2 bottom edge - 3/4 of ply then 1-1/4 into 3-1/2 of joist. Rev AT: the panel had NO connection row of any kind before this.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_face -&gt; deck_joist_tail</t>
+          <t>loft_ceiling -&gt; rear_ledger</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -5768,14 +7407,14 @@
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>#8 x 2 at 6 in o.c. into the tail's y-50 end face, over z 53.75-57.25 - the other half of the notch splice, into the joist sistered to the ledger (Rev AT)</t>
+          <t>construction adhesive + #8 x 2 at 8 in o.c. into the ledger's bottom edge</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_inner -&gt; beam</t>
+          <t>loft_ceiling -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
@@ -5788,14 +7427,14 @@
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL. Rev AT: finish fixing only - this panel starts at z 58, 3/4 above the notch corner, so it does no structural work and is not part of the splice. It had no connection row either.</t>
+          <t>construction adhesive + #8 x 2 at 6 in o.c. into the ledger's bottom edge over the whole 50. Rev AT: tighter than the 8 in field spacing because this is the anchored side of the notch tie - see the beam row below.</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_top -&gt; beam</t>
+          <t>loft_ceiling -&gt; deck_joist_tail</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -5803,39 +7442,39 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL, between the slats. The cap is finish stock doing structural work - it is the slats' seat - so it is fixed on its own account, not by the slat screws alone.</t>
+          <t>construction adhesive + 2 x #8 x 2 into the tail's 1-3/4 of bottom edge, the other anchored side of the notch tie (Rev AT)</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>slat[*] -&gt; beam_wrap_top</t>
+          <t>loft_ceiling -&gt; beam</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>1 x #8 x 3 through the cap into the LVL — 3/4 of cap, 2-1/4 into the beam. Rev AG settles what Rev T left open. slat[22] is the one exception - see below.</t>
+          <t>construction adhesive + #8 x 2 at 6 in o.c. into the beam's bottom edge over x 3 to 27, then 12 in o.c. beyond. Rev AT: this is the SECOND notch restraint, and it acts in the direction the notch would actually fail. A split from the corner at x 3, z 57.25 runs in +x along the grain, and the piece it separates is the beam's bottom 3-1/2 beyond x 3 - whose bottom face is this z 53.75 line. The same sheet is screwed to side_ledger and deck_joist_tail on the other side of x 3, both solidly bearing, so it is a continuous tie holding that piece up against members that cannot move. It is SECONDARY to beam_wrap_face, which is in the plane of the split and works in shear; this works in screw withdrawal from a 1-3/4 landing that is the LVL's LAMINATED EDGE - screws there cross glue lines, so use the stated spacing, do not over-torque, and do not treat this as the primary. Both go on late, so neither is present while the loft is being framed.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>slat[22] -&gt; beam_wrap_top</t>
+          <t>beam_wrap_face -&gt; beam</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -5843,19 +7482,19 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>1 x #8 x 3, OFFSET INBOARD. slat[22] runs x 105.5 to 107 and the LVL ends at 106.25, so only 3/4 of its 1-1/2 width has beam under the cap - the rest is over beam_end_cap, 3/4 ply. A centred screw lands half in ply. Found by the kernel ray cast.</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. in two rows into the LVL - 3/4 of ply then 1-1/4 into 1-3/4 of beam. Rev AT: OVER x 0 TO 27 THIS IS STRUCTURAL, not a finish fixing: tighten to 6 in o.c. in two rows and glue the full contact area. This panel is the notch reinforcement (see beam_tongue) - it straddles the re-entrant corner at x 3, z 57.25 and runs the full length past the shoulder, so it carries across the corner in shear what the LVL would otherwise carry in cross-grain tension. Keep every screw at least 1 in clear of the corner and out of the notch void below z 57.25 at x 0-3. Rev AT: the wrap had no connection row at all before this - its fixing was never specified and never checked.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>ledge_cleat -&gt; wall:bed</t>
+          <t>beam_wrap_face -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
@@ -5863,23 +7502,23 @@
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws into every stud — it carries half an 8 wide lid and whatever is set on it, so it is fixed like a ledger, not tacked like trim</t>
+          <t>#8 x 2 at 6 in o.c. into the ledger's y-50 end face, over z 53.75-57.25. Rev AT: part of the notch splice - this is what ties the tongue back to the member it bears on. End-grain withdrawal is poor and irrelevant here: the joint works in shear.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>ledge_strut[*] -&gt; ledge_cleat</t>
+          <t>beam_wrap_face -&gt; deck_joist_tail</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
@@ -5888,18 +7527,18 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>2 x #8 x 2-1/2 toe-driven into the cleat, plus adhesive</t>
+          <t>#8 x 2 at 6 in o.c. into the tail's y-50 end face, over z 53.75-57.25 - the other half of the notch splice, into the joist sistered to the ledger (Rev AT)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>ledge_strut[*] -&gt; ledge_front_rail</t>
+          <t>beam_wrap_inner -&gt; beam</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C67" s="3" t="inlineStr">
         <is>
@@ -5908,18 +7547,18 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>adhesive + 2 pocket screws from inside the well, angled out of the strut into the back of the rail. Pocket, not toe: a toe screw into 3/4 of poplar from behind breaks out the face, and a screw through the rail's face lands in the strut's end grain.</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL. Rev AT: finish fixing only - this panel starts at z 58, 3/4 above the notch corner, so it does no structural work and is not part of the splice. It had no connection row either.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_strut[*]</t>
+          <t>beam_wrap_top -&gt; beam</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
@@ -5928,18 +7567,18 @@
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4, 2 per strut, countersunk and filled</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL, between the slats. The cap is finish stock doing structural work - it is the slats' seat - so it is fixed on its own account, not by the slat screws alone.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_cleat</t>
+          <t>slat[*] -&gt; beam_wrap_top</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
@@ -5948,14 +7587,14 @@
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4 at 12 in o.c., countersunk and filled — the lid is fixed, not hinged</t>
+          <t>1 x #8 x 3 through the cap into the LVL — 3/4 of cap, 2-1/4 into the beam. Rev AG settles what Rev T left open. slat[22] is the one exception - see below.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>ledge_cleat_rail -&gt; ledge_front_rail</t>
+          <t>slat[22] -&gt; beam_wrap_top</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -5963,19 +7602,19 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-1/4 at 12 in o.c. from inside the well, through the cleat into the rail — screwed from the back so nothing shows on the face</t>
+          <t>1 x #8 x 3, OFFSET INBOARD. slat[22] runs x 105.5 to 107 and the LVL ends at 106.25, so only 3/4 of its 1-1/2 width has beam under the cap - the rest is over beam_end_cap, 3/4 ply. A centred screw lands half in ply. Found by the kernel ray cast.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>ledge_cleat_rail -&gt; deck_ply</t>
+          <t>ledge_cleat -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B71" s="3" t="n">
@@ -5983,43 +7622,43 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #10 x 3-1/2 down through the cleat and the ply into a joist at each of the 9 joists, and #8 x 2 into the ply between them</t>
+          <t>2 x 3 in screws into every stud — it carries half an 8 wide lid and whatever is set on it, so it is fixed like a ledger, not tacked like trim</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_front_rail</t>
+          <t>ledge_strut[*] -&gt; ledge_cleat</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4 at 12 in o.c. into the rail's 3/4 top edge, countersunk and filled. Rev AM: the lid is fixed, never hinged, so this joint is permanent - and with the three struts holding the rail's top on 7.25 it is a flush line the whole 106 1/4, not a joint that has to be pulled closed at assembly.</t>
+          <t>2 x #8 x 2-1/2 toe-driven into the cleat, plus adhesive</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>ledge_rail_splice -&gt; ledge_front_rail</t>
+          <t>ledge_strut[*] -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
@@ -6028,18 +7667,18 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-1/4 at 6 in o.c. in two rows, from inside the well through the splice into the back of both rail pieces - 1/2 into the rail's 3/4</t>
+          <t>adhesive + 2 pocket screws from inside the well, angled out of the strut into the back of the rail. Pocket, not toe: a toe screw into 3/4 of poplar from behind breaks out the face, and a screw through the rail's face lands in the strut's end grain.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_end_cap</t>
+          <t>ledge_lid -&gt; ledge_strut[*]</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
@@ -6048,18 +7687,18 @@
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4, 2 off — the 3/4 x 8 of skirt top edge the lid laps at the stair end (Rev AH)</t>
+          <t>#8 x 1-1/4, 2 per strut, countersunk and filled</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>screen_top_plate -&gt; slat[*]</t>
+          <t>ledge_lid -&gt; ledge_cleat</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C75" s="3" t="inlineStr">
         <is>
@@ -6068,14 +7707,14 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + 1 x #8 x 2-1/2 angled up through the slat into the plate, driven from the loft side, countersunk and filled; 2 x 1-1/2 16ga pins each slat to hold it while the adhesive cures. Rev AS: was UNSPECIFIED. 16ga alone was proposed and is not enough - the structure table calls this screen the GUARD for a 58 deck, and the ceiling note says a 200 lb lean at its top overloads the slat bases. One real screw per slat at each end (the base already has #8 x 3 into the LVL) makes the top a positive connection; the pins are for assembly, not for load.</t>
+          <t>#8 x 1-1/4 at 12 in o.c., countersunk and filled — the lid is fixed, not hinged</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>screen_top_plate -&gt; ceiling</t>
+          <t>ledge_cleat_rail -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
@@ -6083,19 +7722,19 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>into ceiling framing / blocking — joist location not yet measured</t>
+          <t>construction adhesive + #8 x 1-1/4 at 12 in o.c. from inside the well, through the cleat into the rail — screwed from the back so nothing shows on the face</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>lnd_ledger_bedwall -&gt; wall:bed</t>
+          <t>ledge_cleat_rail -&gt; deck_ply</t>
         </is>
       </c>
       <c r="B77" s="3" t="n">
@@ -6103,19 +7742,19 @@
       </c>
       <c r="C77" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>3/8 x 4 lags, 2 per stud</t>
+          <t>construction adhesive + #10 x 3-1/2 down through the cleat and the ply into a joist at each of the 9 joists, and #8 x 2 into the ply between them</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>stringer_b -&gt; lnd_rim</t>
+          <t>ledge_lid -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -6123,19 +7762,19 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>3 x 1/4 x 3-1/2 SDS from inside the box through the rim, before the deck goes on</t>
+          <t>#8 x 1-1/4 at 12 in o.c. into the rail's 3/4 top edge, countersunk and filled. Rev AM: the lid is fixed, never hinged, so this joint is permanent - and with the three struts holding the rail's top on 7.25 it is a flush line the whole 106 1/4, not a joint that has to be pulled closed at assembly.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; lnd_ledger_rightwall</t>
+          <t>ledge_rail_splice -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B79" s="3" t="n">
@@ -6148,14 +7787,14 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>plumb cut on the ledger end + 4 x 1/4 x 4-1/2 SDS into right-wall studs</t>
+          <t>construction adhesive + #8 x 1-1/4 at 6 in o.c. in two rows, from inside the well through the splice into the back of both rail pieces - 1/2 into the rail's 3/4</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_header</t>
+          <t>ledge_lid -&gt; ledge_end_cap</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
@@ -6163,39 +7802,39 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>4 x 1/4 x 3-1/2 SDS over y 18-27. Rev AE: the stringer is on the framing now, not on 3/4 of ply, so a 3-1/2 buries 2 in the header.</t>
+          <t>#8 x 1-1/4, 2 off — the 3/4 x 8 of skirt top edge the lid laps at the stair end (Rev AH)</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_king_b</t>
+          <t>screen_top_plate -&gt; slat[*]</t>
         </is>
       </c>
       <c r="B81" s="3" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS</t>
+          <t>construction adhesive + 1 x #8 x 2-1/2 angled up through the slat into the plate, driven from the loft side, countersunk and filled; 2 x 1-1/2 16ga pins each slat to hold it while the adhesive cures. Rev AS: was UNSPECIFIED. 16ga alone was proposed and is not enough - the structure table calls this screen the GUARD for a 58 deck, and the ceiling note says a 200 lb lean at its top overloads the slat bases. One real screw per slat at each end (the base already has #8 x 3 into the LVL) makes the top a positive connection; the pins are for assembly, not for load.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_trimmer_b</t>
+          <t>screen_top_plate -&gt; ceiling</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -6203,19 +7842,19 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS. Rev AE: the stringer crosses the far jamb pack over z 12-24, so it catches the trimmer as well as the king.</t>
+          <t>into ceiling framing / blocking — joist location not yet measured</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>hw_rake_nailer -&gt; stringer_a</t>
+          <t>lnd_ledger_bedwall -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B83" s="3" t="n">
@@ -6223,19 +7862,19 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + 6 x 3 in screws toe-driven through the nailer into the stringer's face. Rev AE: the nailer's raked end (1-1/2 x 30 on the slope) dies straight onto stringer A now that the sheathing between them is gone.</t>
+          <t>3/8 x 4 lags, 2 per stud</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>lnd_rim -&gt; hw_header</t>
+          <t>stringer_b -&gt; lnd_rim</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -6243,19 +7882,19 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>HUC28 concealed-flange hanger, SD10212 screws straight into the header (flanges would foul the side member on an LUS). Rev AE: no 3/4 facing in the path.</t>
+          <t>3 x 1/4 x 3-1/2 SDS from inside the box through the rim, before the deck goes on</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>lnd_rim -&gt; lnd_ledger_rightwall</t>
+          <t>stringer_c -&gt; lnd_ledger_rightwall</t>
         </is>
       </c>
       <c r="B85" s="3" t="n">
@@ -6263,59 +7902,59 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>HUC28 concealed-flange hanger (an LUS flange would hang past the ledger end)</t>
+          <t>plumb cut on the ledger end + 4 x 1/4 x 4-1/2 SDS into right-wall studs</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>lnd_joist[*] -&gt; lnd_ledger_bedwall</t>
+          <t>stringer_a -&gt; hw_header</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>LUS24</t>
+          <t>4 x 1/4 x 3-1/2 SDS over y 18-27. Rev AE: the stringer is on the framing now, not on 3/4 of ply, so a 3-1/2 buries 2 in the header.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>lnd_joist[*] -&gt; lnd_rim</t>
+          <t>stringer_a -&gt; hw_king_b</t>
         </is>
       </c>
       <c r="B87" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>LUS24 on the rim's back face</t>
+          <t>2 x 1/4 x 3-1/2 SDS</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; lnd_rim</t>
+          <t>stringer_a -&gt; hw_trimmer_b</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
@@ -6328,14 +7967,14 @@
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>2 x A35 at the inside corner, installed before the joists</t>
+          <t>2 x 1/4 x 3-1/2 SDS. Rev AE: the stringer crosses the far jamb pack over z 12-24, so it catches the trimmer as well as the king.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; lnd_rim</t>
+          <t>hw_rake_nailer -&gt; stringer_a</t>
         </is>
       </c>
       <c r="B89" s="3" t="n">
@@ -6348,43 +7987,163 @@
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS toe-screwed from the stringer's outer face; the side member blocks access from inside the box</t>
+          <t>construction adhesive + 6 x 3 in screws toe-driven through the nailer into the stringer's face. Rev AE: the nailer's raked end (1-1/2 x 30 on the slope) dies straight onto stringer A now that the sheathing between them is gone.</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
+          <t>lnd_rim -&gt; hw_header</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>HUC28 concealed-flange hanger, SD10212 screws straight into the header (flanges would foul the side member on an LUS). Rev AE: no 3/4 facing in the path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
+        <is>
+          <t>lnd_rim -&gt; lnd_ledger_rightwall</t>
+        </is>
+      </c>
+      <c r="B91" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C91" s="3" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D91" s="3" t="inlineStr">
+        <is>
+          <t>HUC28 concealed-flange hanger (an LUS flange would hang past the ledger end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>lnd_joist[*] -&gt; lnd_ledger_bedwall</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>LUS24</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="3" t="inlineStr">
+        <is>
+          <t>lnd_joist[*] -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B93" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C93" s="3" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D93" s="3" t="inlineStr">
+        <is>
+          <t>LUS24 on the rim's back face</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>lnd_side_member -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C94" s="2" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>2 x A35 at the inside corner, installed before the joists</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
+        <is>
+          <t>stringer_a -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B95" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C95" s="3" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D95" s="3" t="inlineStr">
+        <is>
+          <t>2 x 1/4 x 3-1/2 SDS toe-screwed from the stringer's outer face; the side member blocks access from inside the box</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
           <t>lnd_blocking[*] -&gt; stringer_b</t>
         </is>
       </c>
-      <c r="B90" s="2" t="n">
+      <c r="B96" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="C90" s="2" t="inlineStr">
+      <c r="C96" s="2" t="inlineStr">
         <is>
           <t>face-screw</t>
         </is>
       </c>
-      <c r="D90" s="2" t="inlineStr">
+      <c r="D96" s="2" t="inlineStr">
         <is>
           <t>2 x 3 in screws each end, toe-driven</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D90"/>
+  <autoFilter ref="A1:D96"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6417,7 +8176,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated from dimensions.yaml rev AU</t>
+          <t>Generated from dimensions.yaml rev AX</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -6429,17 +8188,17 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>GRADE</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Every species/grade cell says TBD</t>
+          <t>Deck and ceiling ply layouts, chosen for joinery (Rev AX)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Pending price and availability. Three ply grades are needed and they are not interchangeable: structural (deck_ply, the half-wall sheathing), paint-grade show faces (beam wrap, ledge rail and lid, treads, risers, nook lining), and 1/2 flitches (jamb packs, the header's middle ply).</t>
+          <t>The deck is THREE pieces: two rows to x 62 1/4 either side of a blocked cross-joist seam at y 24, then one full-depth 44 x 48 1/4 panel over the landing end with no seam in it — the part walked on rather than slept on. Both seams sit under the mattress; the long one lands on joist 5 and needs no blocking. 62 1/4 is the furthest in it can go: the next joist would need a 56 wide panel against a 48 sheet width. The ceiling is three pieces with BOTH seams on joist centres (38 1/4, 74 1/4), so every ceiling seam is backed. Trimming the deck to a flat 48 was considered and rejected — it changed no sheet count and would have left beam_wrap_inner's foot over a 1/4 void. COST, stated plainly: these layouts are 9 sheets at 64%. The cheapest nest was 7 at 83%, with a full-width deck seam and a cross-joist seam in the ceiling. Two sheets bought better joinery, knowingly.</t>
         </is>
       </c>
     </row>
@@ -6451,63 +8210,63 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Deck-ply front-edge blocking is now in the model (Rev AU)</t>
+          <t>The loft deck IS the finished walking surface (2026-09-07)</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Nine 2x4 blocks on edge at the beam face — eight at 10 1/2 on a 12 pitch plus one 5 3/4 at the rim, all from one 8 ft board, and they are counted in the Buy list and the Cut list. Fixed with 2 x 1/4 x 3 per block driven from the beam's OUTBOARD face before beam_wrap_face closes it, then the ply glued and screwed down onto them at 6 in o.c. SEQUENCE: before the deck ply.</t>
+          <t>It decides the deck's grade, which is why it matters here. The mattress covers y 8 3/4 to 46 3/4 out to about x 77; the rest is walked on and nothing in the model covers it. If it is the finished floor it wants a sanded, paintable face and sealed edges rather than rated sheathing — and the whole 3 sheets move to the paint-grade group. Nesting is indifferent: 3/4 ply comes to the same 10 sheets whether it is bought as one pool or split by grade, so this is purely about the product and the price, not the quantity.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>CLOSED</t>
+          <t>GRADE</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>The beam notch needs no separate ply cheek (Rev AT)</t>
+          <t>Every species/grade cell says TBD</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>It is beam_wrap_face, which already spans the corner on the clear outboard face: adhesive + #8 x 2 at 6 in o.c. over x 0-27, into the tongue above z 57 1/4 and into the ledger and joist-tail end faces below it. Nothing extra to buy — but the wrap's fixing over that first 27 in is STRUCTURAL, not finish, and its screws must stay 1 in clear of the corner and out of the notch void below z 57 1/4.</t>
+          <t>Pending price and availability. Three ply grades are needed and they are not interchangeable: structural (deck_ply, the half-wall sheathing), paint-grade show faces (beam wrap, ledge rail and lid, treads, risers, nook lining), and 1/2 flitches (jamb packs, the header's middle ply).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>FIELD</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Stud locations: bed wall, window wall, right wall</t>
+          <t>Deck-ply front-edge blocking is now in the model (Rev AU)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Every ledger fixing count on the Hardware tab assumes 16 in o.c. The window wall needs a stud (or added blocking) within ~6 in of y 50 for the beam's end reaction.</t>
+          <t>Nine 2x4 blocks on edge at the beam face — eight at 10 1/2 on a 12 pitch plus one 5 3/4 at the rim, all from one 8 ft board, and they are counted in the Buy list and the Cut list. Fixed with 2 x 1/4 x 3 per block driven from the beam's OUTBOARD face before beam_wrap_face closes it, then the ply glued and screwed down onto them at 6 in o.c. SEQUENCE: before the deck ply.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>FIELD</t>
+          <t>CLOSED</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Ceiling joist nearest 50 3/4 from the bed wall</t>
+          <t>The beam notch needs no separate ply cheek (Rev AT)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>No longer gates the design (Rev AS: the plate is fixed at 47 1/4-50 3/4 and blocking can be added from the attic), but it decides whether you screw to a joist or block first.</t>
+          <t>It is beam_wrap_face, which already spans the corner on the clear outboard face: adhesive + #8 x 2 at 6 in o.c. over x 0-27, into the tongue above z 57 1/4 and into the ledger and joist-tail end faces below it. Nothing extra to buy — but the wrap's fixing over that first 27 in is STRUCTURAL, not finish, and its screws must stay 1 in clear of the corner and out of the notch void below z 57 1/4.</t>
         </is>
       </c>
     </row>
@@ -6519,44 +8278,44 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Floor joists under the half-wall plate and the kicker</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr"/>
+          <t>Stud locations: bed wall, window wall, right wall</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Every ledger fixing count on the Hardware tab assumes 16 in o.c. The window wall needs a stud (or added blocking) within ~6 in of y 50 for the beam's end reaction.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>SPECIFY</t>
+          <t>FIELD</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>hw_bottom_plate_a / _b to floor</t>
+          <t>Ceiling joist nearest 50 3/4 from the bed wall</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Left TBD by the user 2026-09-06.</t>
+          <t>No longer gates the design (Rev AS: the plate is fixed at 47 1/4-50 3/4 and blocking can be added from the attic), but it decides whether you screw to a joist or block first.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>CHECKER</t>
+          <t>FIELD</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>10 connections carry NO fastener key at all</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Filter the Hardware tab for 'NO FASTENER KEY'. verify.py only reports a row that literally says UNSPECIFIED, so these pass silently: beam -&gt; hw_top_plate_2; deck_rim -&gt; hw_top_plate_2; hw_header -&gt; hw_trimmer_a; hw_header -&gt; hw_trimmer_b; hw_top_plate_1 -&gt; hw_header; hw_top_plate_1 -&gt; hw_king_a; hw_top_plate_1 -&gt; hw_king_b; stringer_a -&gt; kicker; stringer_b -&gt; kicker; stringer_c -&gt; kicker. Most are ordinary nailing, but the kicker is already an open anchorage item. Worth making verify.py WARN on a missing key — it would change the 0 WARN baseline, so it is your call. (Counted from the model, not typed: an earlier hand count said 8.)</t>
-        </is>
-      </c>
+          <t>Floor joists under the half-wall plate and the kicker</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -6566,47 +8325,81 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>kicker anchorage</t>
-        </is>
-      </c>
-      <c r="C11" s="3" t="inlineStr"/>
+          <t>hw_bottom_plate_a / _b to floor</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Left TBD by the user 2026-09-06.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>METHOD</t>
+          <t>CHECKER</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Sheet counts are shelf-packed, not nested</t>
+          <t>10 connections carry NO fastener key at all</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>The Sheet goods tab lists every panel with its real size. Buy the counts as a floor, not a ceiling, and lay out the deck and the loft ceiling on paper first: both are OVER 48 in y (48 1/4 and 50), so that dimension has to run along the sheet's 8 ft length and each takes one sheet per piece.</t>
+          <t>Filter the Hardware tab for 'NO FASTENER KEY'. verify.py only reports a row that literally says UNSPECIFIED, so these pass silently: beam -&gt; hw_top_plate_2; deck_rim -&gt; hw_top_plate_2; hw_header -&gt; hw_trimmer_a; hw_header -&gt; hw_trimmer_b; hw_top_plate_1 -&gt; hw_header; hw_top_plate_1 -&gt; hw_king_a; hw_top_plate_1 -&gt; hw_king_b; stringer_a -&gt; kicker; stringer_b -&gt; kicker; stringer_c -&gt; kicker. Most are ordinary nailing, but the kicker is already an open anchorage item. Worth making verify.py WARN on a missing key — it would change the 0 WARN baseline, so it is your call. (Counted from the model, not typed: an earlier hand count said 8.)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
+          <t>SPECIFY</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>kicker anchorage</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr">
+        <is>
           <t>METHOD</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Sheet counts are shelf-packed, not nested</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>The Sheet goods tab lists every panel with its real size. Buy the counts as a floor, not a ceiling, and lay out the deck and the loft ceiling on paper first: both are OVER 48 in y (48 1/4 and 50), so that dimension has to run along the sheet's 8 ft length and each takes one sheet per piece.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>METHOD</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>Cut lengths are FRAMING extents</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>Finished faces are their own parts. No waste allowance is added anywhere; the board counts include a 1/8 kerf per cut and nothing else.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C13"/>
+  <autoFilter ref="A1:C15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Rev AY: drawing-auditor and connection-checker run
</commit_message>
<xml_diff>
--- a/materials/materials-list.xlsx
+++ b/materials/materials-list.xlsx
@@ -19,7 +19,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Cut list'!$A$1:$I$58</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Sheet goods'!$A$1:$F$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Cut layout'!$A$1:$I$41</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Hardware'!$A$1:$D$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Hardware'!$A$1:$D$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'TBD and assumptions'!$A$1:$C$15</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2392,7 +2392,7 @@
       </c>
       <c r="I36" s="2" t="inlineStr">
         <is>
-          <t>CUT AS 3 PIECES: 62¼×24 + 62¼×24¼ + 44×48¼ — two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
+          <t>CUT AS 3 PIECES: 62¼×24 + 62¼×24¼ + 44×48¼ — two rows to x 62¼ either side of the y-24 seam, then one full-depth 44 x 48¼ panel over the landing end; seam on joist 5's centre — all derived from the blocking</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
+          <t>two rows to x 62¼ either side of the y-24 seam, then one full-depth 44 x 48¼ panel over the landing end; seam on joist 5's centre — all derived from the blocking</t>
         </is>
       </c>
     </row>
@@ -3557,7 +3557,7 @@
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
+          <t>two rows to x 62¼ either side of the y-24 seam, then one full-depth 44 x 48¼ panel over the landing end; seam on joist 5's centre — all derived from the blocking</t>
         </is>
       </c>
     </row>
@@ -4085,7 +4085,7 @@
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>two rows to x 62 1/4 either side of the y-24 seam, then one full-depth 44 x 48 1/4 panel over the landing end; long seam on joist 5's centre, 14 3/4 inside the mattress edge</t>
+          <t>two rows to x 62¼ either side of the y-24 seam, then one full-depth 44 x 48¼ panel over the landing end; seam on joist 5's centre — all derived from the blocking</t>
         </is>
       </c>
     </row>
@@ -6226,7 +6226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D96"/>
+  <dimension ref="A1:D103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -6264,7 +6264,7 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
@@ -6338,7 +6338,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
@@ -6427,7 +6427,7 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3 structural screws per block, driven from the beam's OUTBOARD face at y 50 through 1 3/4 of LVL and 1 1/4 into the block. Rev AU: preferred over toe-screwing from inside the bay because it puts the fastener in shear instead of relying on a toed screw, and the y-50 face is open until beam_wrap_face goes on - the heads end up behind the wrap. SEQUENCE: before the wrap, and before the deck ply.</t>
+          <t>2 x 1/4 x 3 structural screws per block at z 54 1/4 and 56 3/4, driven from the beam's OUTBOARD face at y 50 through 1 3/4 of LVL and 1 1/4 into the block. Rev AY: the z is stated because beam_wrap_face's structural rows come through the same face at the same x stations - keep them off each other. Rev AU: preferred over toe-screwing from inside the bay because it puts the fastener in shear instead of relying on a toed screw, and the y-50 face is open until beam_wrap_face goes on - the heads end up behind the wrap. SEQUENCE: before the wrap, and before the deck ply.</t>
         </is>
       </c>
     </row>
@@ -6507,14 +6507,14 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[0] here and deck_joist[1] at the far end, which carries no row of its own</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[0]</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>deck_seam_blocking[1] -&gt; deck_joist[1]</t>
+          <t>deck_seam_blocking[0] -&gt; deck_joist[1]</t>
         </is>
       </c>
       <c r="B16" s="2" t="n">
@@ -6527,14 +6527,14 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[1] here and deck_joist[2] at the far end, which carries no row of its own</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[1]. Rev AY: the far end used to be asserted in the other row's note and never checked. The block has no bearing shelf - it hangs at z 55.75-57.25 on toe-screws at BOTH ends - so both ends carry, and both are now declared.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>deck_seam_blocking[2] -&gt; deck_joist[2]</t>
+          <t>deck_seam_blocking[1] -&gt; deck_joist[1]</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
@@ -6547,14 +6547,14 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[2] here and deck_joist[3] at the far end, which carries no row of its own</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[1]</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>deck_seam_blocking[3] -&gt; deck_joist[3]</t>
+          <t>deck_seam_blocking[1] -&gt; deck_joist[2]</t>
         </is>
       </c>
       <c r="B18" s="2" t="n">
@@ -6567,14 +6567,14 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[3] here and deck_joist[4] at the far end, which carries no row of its own</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[2]. Rev AY: the far end used to be asserted in the other row's note and never checked. The block has no bearing shelf - it hangs at z 55.75-57.25 on toe-screws at BOTH ends - so both ends carry, and both are now declared.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>deck_seam_blocking[4] -&gt; deck_joist[4]</t>
+          <t>deck_seam_blocking[2] -&gt; deck_joist[2]</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -6587,34 +6587,34 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven at EACH end - into deck_joist[4] here and deck_joist[5] at the far end, which carries no row of its own</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[2]</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>deck_ply -&gt; deck_seam_blocking[*]</t>
+          <t>deck_seam_blocking[2] -&gt; deck_joist[3]</t>
         </is>
       </c>
       <c r="B20" s="2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. through BOTH panel edges - the seam is a butt joint in the deck diaphragm and both sides land on this block (Rev AV)</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[3]. Rev AY: the far end used to be asserted in the other row's note and never checked. The block has no bearing shelf - it hangs at z 55.75-57.25 on toe-screws at BOTH ends - so both ends carry, and both are now declared.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>deck_ply -&gt; side_ledger</t>
+          <t>deck_seam_blocking[3] -&gt; deck_joist[3]</t>
         </is>
       </c>
       <c r="B21" s="3" t="n">
@@ -6622,19 +6622,19 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. — structural, not just an edge fixing, because the ply diaphragm is what keeps the shallow ledger from rolling under the beam's eccentric load</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[3]</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>deck_ply -&gt; rear_ledger</t>
+          <t>deck_seam_blocking[3] -&gt; deck_joist[4]</t>
         </is>
       </c>
       <c r="B22" s="2" t="n">
@@ -6642,19 +6642,19 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c., same as the side ledger — Rev AO drops rear_ledger to deck level so the ply runs over its top the same way</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[4]. Rev AY: the far end used to be asserted in the other row's note and never checked. The block has no bearing shelf - it hangs at z 55.75-57.25 on toe-screws at BOTH ends - so both ends carry, and both are now declared.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>beam -&gt; hw_top_plate_2</t>
+          <t>deck_seam_blocking[4] -&gt; deck_joist[4]</t>
         </is>
       </c>
       <c r="B23" s="3" t="n">
@@ -6662,19 +6662,19 @@
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[4]</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>deck_rim -&gt; hw_top_plate_2</t>
+          <t>deck_seam_blocking[4] -&gt; deck_joist[5]</t>
         </is>
       </c>
       <c r="B24" s="2" t="n">
@@ -6682,39 +6682,39 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>2 x 3 in screws toe-driven into deck_joist[5]. Rev AY: the far end used to be asserted in the other row's note and never checked. The block has no bearing shelf - it hangs at z 55.75-57.25 on toe-screws at BOTH ends - so both ends carry, and both are now declared.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>rear_ledger -&gt; wall:bed</t>
+          <t>deck_ply -&gt; deck_seam_blocking[*]</t>
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>3/8 x 4 lags, 2 per stud staggered, into every stud - the same fastener as lnd_ledger_bedwall. Rev AS: was the sizeless 'lags into every stud'. 1 1/2 of 2x4 ledger + 5/8 of board = 2 1/8 crossed, 1 7/8 of embedment.</t>
+          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. through BOTH panel edges - the seam is a butt joint in the deck diaphragm and both sides land on this block (Rev AV)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>side_ledger -&gt; wall:window</t>
+          <t>deck_ply -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B26" s="2" t="n">
@@ -6722,19 +6722,19 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>1/4 x 4 structural screws, 2 per stud staggered top and bottom, plus a pair within 6 in of y 50 — FIELD, confirm a stud lands there or add blocking in the wall</t>
+          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c. — structural, not just an edge fixing, because the ply diaphragm is what keeps the shallow ledger from rolling under the beam's eccentric load</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>hw_header -&gt; hw_trimmer_a</t>
+          <t>deck_ply -&gt; rear_ledger</t>
         </is>
       </c>
       <c r="B27" s="3" t="n">
@@ -6747,14 +6747,14 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>construction adhesive + #8 x 1-5/8 at 6 in o.c., same as the side ledger — Rev AO drops rear_ledger to deck level so the ply runs over its top the same way</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>hw_header -&gt; hw_trimmer_b</t>
+          <t>beam -&gt; hw_top_plate_2</t>
         </is>
       </c>
       <c r="B28" s="2" t="n">
@@ -6774,7 +6774,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>hw_jamb_ply_a -&gt; hw_bottom_plate_a</t>
+          <t>deck_rim -&gt; hw_top_plate_2</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
@@ -6787,14 +6787,14 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>bears with the trimmer; held by the pack nailing below</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>hw_jamb_ply_b -&gt; hw_bottom_plate_b</t>
+          <t>rear_ledger -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B30" s="2" t="n">
@@ -6802,19 +6802,19 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>bears with the trimmer; held by the pack nailing below</t>
+          <t>3/8 x 4 lags, 2 per stud staggered, into every stud - the same fastener as lnd_ledger_bedwall. Rev AS: was the sizeless 'lags into every stud'. 1 1/2 of 2x4 ledger + 5/8 of board = 2 1/8 crossed, 1 7/8 of embedment.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>hw_trimmer_a -&gt; hw_king_a</t>
+          <t>side_ledger -&gt; wall:window</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
@@ -6822,19 +6822,19 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
+          <t>1/4 x 4 structural screws, 2 per stud staggered top and bottom, plus a pair within 6 in of y 50 — FIELD, confirm a stud lands there or add blocking in the wall</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>hw_trimmer_b -&gt; hw_king_b</t>
+          <t>hw_header -&gt; hw_trimmer_a</t>
         </is>
       </c>
       <c r="B32" s="2" t="n">
@@ -6842,19 +6842,19 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>hw_top_plate_2 -&gt; hw_top_plate_1</t>
+          <t>hw_header -&gt; hw_trimmer_b</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
@@ -6867,14 +6867,14 @@
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>16d at 16 in o.c., staggered — the upper plate laps the lower at the wall's ends</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>hw_king_a -&gt; hw_bottom_plate_a</t>
+          <t>hw_jamb_ply_a -&gt; hw_bottom_plate_a</t>
         </is>
       </c>
       <c r="B34" s="2" t="n">
@@ -6887,14 +6887,14 @@
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate</t>
+          <t>bears with the trimmer; held by the pack nailing below</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>hw_king_b -&gt; hw_bottom_plate_b</t>
+          <t>hw_jamb_ply_b -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
@@ -6907,14 +6907,14 @@
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate. This is the stud the beam's stair-end reaction comes down; Rev AG's connection audit found the post asserted in prose and never declared.</t>
+          <t>bears with the trimmer; held by the pack nailing below</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>hw_top_plate_1 -&gt; hw_header</t>
+          <t>hw_trimmer_a -&gt; hw_king_a</t>
         </is>
       </c>
       <c r="B36" s="2" t="n">
@@ -6922,19 +6922,19 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>hw_top_plate_1 -&gt; hw_king_a</t>
+          <t>hw_trimmer_b -&gt; hw_king_b</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
@@ -6942,19 +6942,19 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>16d nails in two rows at 12 in o.c. + construction adhesive on both faces of the ply — this is what makes the pack act as one 3.5 post</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>hw_top_plate_1 -&gt; hw_king_b</t>
+          <t>hw_top_plate_2 -&gt; hw_top_plate_1</t>
         </is>
       </c>
       <c r="B38" s="2" t="n">
@@ -6967,14 +6967,14 @@
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>16d at 16 in o.c., staggered — the upper plate laps the lower at the wall's ends</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>hw_bottom_plate_a -&gt; floor</t>
+          <t>hw_king_a -&gt; hw_bottom_plate_a</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
@@ -6982,19 +6982,19 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>UNSPECIFIED — declared open</t>
+          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>hw_bottom_plate_b -&gt; floor</t>
+          <t>hw_king_b -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B40" s="2" t="n">
@@ -7002,23 +7002,23 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>UNSPECIFIED — declared open</t>
+          <t>2 x 3 in screws toe-driven, or end-nailed 2 x 16d through the plate. This is the stud the beam's stair-end reaction comes down; Rev AG's connection audit found the post asserted in prose and never declared.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>nk_bedwall_stud[*] -&gt; hw_bottom_plate_a</t>
+          <t>hw_top_plate_1 -&gt; hw_header</t>
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
@@ -7027,18 +7027,18 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven each stud</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>nk_bedwall_cap -&gt; nk_bedwall_stud[*]</t>
+          <t>hw_top_plate_1 -&gt; hw_king_a</t>
         </is>
       </c>
       <c r="B42" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
@@ -7047,14 +7047,14 @@
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws through the cap into each stud</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>lnd_ledger_bedwall -&gt; nk_bedwall_cap</t>
+          <t>hw_top_plate_1 -&gt; hw_king_b</t>
         </is>
       </c>
       <c r="B43" s="3" t="n">
@@ -7067,14 +7067,14 @@
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>3 in screws up through the cap into the ledger at each stud — secondary only, the ledger's own load path is its lags into the bed-wall studs</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>lnd_ledger_rightwall -&gt; nk_bedwall_cap</t>
+          <t>hw_bottom_plate_a -&gt; floor</t>
         </is>
       </c>
       <c r="B44" s="2" t="n">
@@ -7082,19 +7082,19 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>3 in screws up through the cap, at the cap's right-hand end</t>
+          <t>UNSPECIFIED — declared open</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; nk_bedwall_cap</t>
+          <t>hw_bottom_plate_b -&gt; floor</t>
         </is>
       </c>
       <c r="B45" s="3" t="n">
@@ -7102,19 +7102,19 @@
       </c>
       <c r="C45" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D45" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws up through the cap into the side member</t>
+          <t>UNSPECIFIED — declared open</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>nk_shortwall_strut[*] -&gt; hw_bottom_plate_b</t>
+          <t>nk_bedwall_stud[*] -&gt; hw_bottom_plate_a</t>
         </is>
       </c>
       <c r="B46" s="2" t="n">
@@ -7127,34 +7127,34 @@
       </c>
       <c r="D46" s="2" t="inlineStr">
         <is>
-          <t>2 x 3 in screws toe-driven each strut</t>
+          <t>2 x 3 in screws toe-driven each stud</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>hw_rake_nailer -&gt; hw_trimmer_b</t>
+          <t>nk_bedwall_cap -&gt; nk_bedwall_stud[*]</t>
         </is>
       </c>
       <c r="B47" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C47" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D47" s="3" t="inlineStr">
         <is>
-          <t>3 x 3 in screws through the trimmer into the nailer's end</t>
+          <t>2 x 3 in screws through the cap into each stud</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; hw_header</t>
+          <t>lnd_ledger_bedwall -&gt; nk_bedwall_cap</t>
         </is>
       </c>
       <c r="B48" s="2" t="n">
@@ -7162,19 +7162,19 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>6 × 1/4 × 4 structural screws. Rev AE: direct into the header, no 3/4 facing in the path, so 4 in reaches the depth 5 in used to.</t>
+          <t>3 in screws up through the cap into the ledger at each stud — secondary only, the ledger's own load path is its lags into the bed-wall studs</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>lnd_ledger_rightwall -&gt; wall:right</t>
+          <t>lnd_ledger_rightwall -&gt; nk_bedwall_cap</t>
         </is>
       </c>
       <c r="B49" s="3" t="n">
@@ -7182,19 +7182,19 @@
       </c>
       <c r="C49" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D49" s="3" t="inlineStr">
         <is>
-          <t>1/4 x 4 flat-head structural screws (SDWS22400 or equal), 2 per stud staggered. Rev AS: the wall is 5/8 drywall on wood studs, so a screw crosses 1 1/2 of 2x8 ledger + 5/8 of board = 2 1/8 before it reaches the stud; a 4 leaves 1 7/8 of embedment. Do not substitute 3 1/2 here - that is only 1 3/8 in the stud.</t>
+          <t>3 in screws up through the cap, at the cap's right-hand end</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; wall:right</t>
+          <t>lnd_side_member -&gt; nk_bedwall_cap</t>
         </is>
       </c>
       <c r="B50" s="2" t="n">
@@ -7202,39 +7202,39 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
         <is>
-          <t>1/4 x 4 flat-head structural screws, 2 per stud into every stud the stringer crosses. Rev AS: was the bare Rev T phrase 'fastens to the right wall', which specified nothing. Same 2 1/8 of ledger + board to cross as lnd_ledger_rightwall.</t>
+          <t>2 x 3 in screws up through the cap into the side member</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>stringer_a_skin -&gt; stringer_a</t>
+          <t>nk_shortwall_strut[*] -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B51" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C51" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D51" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + 1-1/2 x 16ga finish nails at 8 in o.c. into the stringer's outer face (3/4 penetration)</t>
+          <t>2 x 3 in screws toe-driven each strut</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; stringer_a_skin</t>
+          <t>hw_rake_nailer -&gt; hw_trimmer_b</t>
         </is>
       </c>
       <c r="B52" s="2" t="n">
@@ -7247,14 +7247,14 @@
       </c>
       <c r="D52" s="2" t="inlineStr">
         <is>
-          <t>1-1/2 x 16ga finish nails at 8 in o.c. through the skin into the cleat, plus adhesive</t>
+          <t>3 x 3 in screws through the trimmer into the nailer's end</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; hw_bottom_plate_b</t>
+          <t>lnd_side_member -&gt; hw_header</t>
         </is>
       </c>
       <c r="B53" s="3" t="n">
@@ -7267,14 +7267,14 @@
       </c>
       <c r="D53" s="3" t="inlineStr">
         <is>
-          <t>2 x #10 x 3 screws through the plate's end into the cleat</t>
+          <t>6 × 1/4 × 4 structural screws. Rev AE: direct into the header, no 3/4 facing in the path, so 4 in reaches the depth 5 in used to.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; stringer_a</t>
+          <t>lnd_ledger_rightwall -&gt; wall:right</t>
         </is>
       </c>
       <c r="B54" s="2" t="n">
@@ -7282,19 +7282,19 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
         <is>
-          <t>adhesive + 3 x #10 x 2-1/2 screws up through the cleat's ripped top into the stringer, over the 5 in of angled contact at its downhill end</t>
+          <t>1/4 x 4 flat-head structural screws (SDWS22400 or equal), 2 per stud staggered. Rev AS: the wall is 5/8 drywall on wood studs, so a screw crosses 1 1/2 of 2x8 ledger + 5/8 of board = 2 1/8 before it reaches the stud; a 4 leaves 1 7/8 of embedment. Do not substitute 3 1/2 here - that is only 1 3/8 in the stud.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>stringer_a_skin_cleat -&gt; floor</t>
+          <t>stringer_c -&gt; wall:right</t>
         </is>
       </c>
       <c r="B55" s="3" t="n">
@@ -7302,19 +7302,19 @@
       </c>
       <c r="C55" s="3" t="inlineStr">
         <is>
-          <t>floor</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D55" s="3" t="inlineStr">
         <is>
-          <t>3 x #10 x 3 screws into the subfloor</t>
+          <t>1/4 x 4 flat-head structural screws, 2 per stud into every stud the stringer crosses. Rev AS: was the bare Rev T phrase 'fastens to the right wall', which specified nothing. Same 2 1/8 of ledger + board to cross as lnd_ledger_rightwall.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; kicker</t>
+          <t>stringer_a_skin -&gt; stringer_a</t>
         </is>
       </c>
       <c r="B56" s="2" t="n">
@@ -7322,19 +7322,19 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>construction adhesive + 1-1/2 x 16ga finish nails at 8 in o.c. into the stringer's outer face (3/4 penetration)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>stringer_b -&gt; kicker</t>
+          <t>stringer_a_skin_cleat -&gt; stringer_a_skin</t>
         </is>
       </c>
       <c r="B57" s="3" t="n">
@@ -7342,19 +7342,19 @@
       </c>
       <c r="C57" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D57" s="3" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>1-1/2 x 16ga finish nails at 8 in o.c. through the skin into the cleat, plus adhesive</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; kicker</t>
+          <t>stringer_a_skin_cleat -&gt; hw_bottom_plate_b</t>
         </is>
       </c>
       <c r="B58" s="2" t="n">
@@ -7362,39 +7362,39 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
         <is>
-          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
+          <t>2 x #10 x 3 screws through the plate's end into the cleat</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; deck_joist[*]</t>
+          <t>stringer_a_skin_cleat -&gt; stringer_a</t>
         </is>
       </c>
       <c r="B59" s="3" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="C59" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D59" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 8 in o.c. up into each joist's 1-1/2 bottom edge - 3/4 of ply then 1-1/4 into 3-1/2 of joist. Rev AT: the panel had NO connection row of any kind before this.</t>
+          <t>adhesive + 3 x #10 x 2-1/2 screws up through the cleat's ripped top into the stringer, over the 5 in of angled contact at its downhill end</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; rear_ledger</t>
+          <t>stringer_a_skin_cleat -&gt; floor</t>
         </is>
       </c>
       <c r="B60" s="2" t="n">
@@ -7402,19 +7402,19 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 8 in o.c. into the ledger's bottom edge</t>
+          <t>3 x #10 x 3 screws into the subfloor</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; side_ledger</t>
+          <t>kicker -&gt; floor</t>
         </is>
       </c>
       <c r="B61" s="3" t="n">
@@ -7422,19 +7422,19 @@
       </c>
       <c r="C61" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>floor</t>
         </is>
       </c>
       <c r="D61" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 6 in o.c. into the ledger's bottom edge over the whole 50. Rev AT: tighter than the 8 in field spacing because this is the anchored side of the notch tie - see the beam row below.</t>
+          <t>UNSPECIFIED — declared open</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; deck_joist_tail</t>
+          <t>stringer_a -&gt; kicker</t>
         </is>
       </c>
       <c r="B62" s="2" t="n">
@@ -7442,19 +7442,19 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + 2 x #8 x 2 into the tail's 1-3/4 of bottom edge, the other anchored side of the notch tie (Rev AT)</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>loft_ceiling -&gt; beam</t>
+          <t>stringer_b -&gt; kicker</t>
         </is>
       </c>
       <c r="B63" s="3" t="n">
@@ -7462,19 +7462,19 @@
       </c>
       <c r="C63" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D63" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 6 in o.c. into the beam's bottom edge over x 3 to 27, then 12 in o.c. beyond. Rev AT: this is the SECOND notch restraint, and it acts in the direction the notch would actually fail. A split from the corner at x 3, z 57.25 runs in +x along the grain, and the piece it separates is the beam's bottom 3-1/2 beyond x 3 - whose bottom face is this z 53.75 line. The same sheet is screwed to side_ledger and deck_joist_tail on the other side of x 3, both solidly bearing, so it is a continuous tie holding that piece up against members that cannot move. It is SECONDARY to beam_wrap_face, which is in the plane of the split and works in shear; this works in screw withdrawal from a 1-3/4 landing that is the LVL's LAMINATED EDGE - screws there cross glue lines, so use the stated spacing, do not over-torque, and do not treat this as the primary. Both go on late, so neither is present while the loft is being framed.</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_face -&gt; beam</t>
+          <t>stringer_c -&gt; kicker</t>
         </is>
       </c>
       <c r="B64" s="2" t="n">
@@ -7482,23 +7482,23 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. in two rows into the LVL - 3/4 of ply then 1-1/4 into 1-3/4 of beam. Rev AT: OVER x 0 TO 27 THIS IS STRUCTURAL, not a finish fixing: tighten to 6 in o.c. in two rows and glue the full contact area. This panel is the notch reinforcement (see beam_tongue) - it straddles the re-entrant corner at x 3, z 57.25 and runs the full length past the shoulder, so it carries across the corner in shear what the LVL would otherwise carry in cross-grain tension. Keep every screw at least 1 in clear of the corner and out of the notch void below z 57.25 at x 0-3. Rev AT: the wrap had no connection row at all before this - its fixing was never specified and never checked.</t>
+          <t>NO FASTENER KEY — silent in verify.py, which only reports the rows that say UNSPECIFIED</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_face -&gt; side_ledger</t>
+          <t>loft_ceiling -&gt; deck_joist[*]</t>
         </is>
       </c>
       <c r="B65" s="3" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="C65" s="3" t="inlineStr">
         <is>
@@ -7507,14 +7507,14 @@
       </c>
       <c r="D65" s="3" t="inlineStr">
         <is>
-          <t>#8 x 2 at 6 in o.c. into the ledger's y-50 end face, over z 53.75-57.25. Rev AT: part of the notch splice - this is what ties the tongue back to the member it bears on. End-grain withdrawal is poor and irrelevant here: the joint works in shear.</t>
+          <t>construction adhesive + #8 x 2 at 8 in o.c. up into each joist's 1-1/2 bottom edge - 3/4 of ply then 1-1/4 into 3-1/2 of joist. Rev AT: the panel had NO connection row of any kind before this.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_face -&gt; deck_joist_tail</t>
+          <t>loft_ceiling -&gt; rear_ledger</t>
         </is>
       </c>
       <c r="B66" s="2" t="n">
@@ -7527,14 +7527,14 @@
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>#8 x 2 at 6 in o.c. into the tail's y-50 end face, over z 53.75-57.25 - the other half of the notch splice, into the joist sistered to the ledger (Rev AT)</t>
+          <t>construction adhesive + #8 x 2 at 8 in o.c. into the ledger's bottom edge</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>beam_wrap_inner -&gt; beam</t>
+          <t>loft_ceiling -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B67" s="3" t="n">
@@ -7547,14 +7547,14 @@
       </c>
       <c r="D67" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL. Rev AT: finish fixing only - this panel starts at z 58, 3/4 above the notch corner, so it does no structural work and is not part of the splice. It had no connection row either.</t>
+          <t>construction adhesive + #8 x 2 at 6 in o.c. into the ledger's bottom edge over the whole 50. Rev AT: tighter than the 8 in field spacing because this is the anchored side of the notch tie - see the beam row below.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>beam_wrap_top -&gt; beam</t>
+          <t>loft_ceiling -&gt; deck_joist_tail</t>
         </is>
       </c>
       <c r="B68" s="2" t="n">
@@ -7562,39 +7562,39 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL, between the slats. The cap is finish stock doing structural work - it is the slats' seat - so it is fixed on its own account, not by the slat screws alone.</t>
+          <t>construction adhesive + 2 x #8 x 2 into the tail's 1-3/4 of bottom edge, the other anchored side of the notch tie (Rev AT)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>slat[*] -&gt; beam_wrap_top</t>
+          <t>loft_ceiling -&gt; beam</t>
         </is>
       </c>
       <c r="B69" s="3" t="n">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="C69" s="3" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D69" s="3" t="inlineStr">
         <is>
-          <t>1 x #8 x 3 through the cap into the LVL — 3/4 of cap, 2-1/4 into the beam. Rev AG settles what Rev T left open. slat[22] is the one exception - see below.</t>
+          <t>construction adhesive + #8 x 2 at 6 in o.c. into the beam's bottom edge over x 3 to 27, then 12 in o.c. beyond. Rev AT: this is the SECOND notch restraint, and it acts in the direction the notch would actually fail. A split from the corner at x 3, z 57.25 runs in +x along the grain, and the piece it separates is the beam's bottom 3-1/2 beyond x 3 - whose bottom face is this z 53.75 line. The same sheet is screwed to side_ledger and deck_joist_tail on the other side of x 3, both solidly bearing, so it is a continuous tie holding that piece up against members that cannot move. It is SECONDARY to beam_wrap_face, which is in the plane of the split and works in shear; this works in screw withdrawal from a 1-3/4 landing that is the LVL's LAMINATED EDGE - screws there cross glue lines, so use the stated spacing, do not over-torque, and do not treat this as the primary. Both go on late, so neither is present while the loft is being framed.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>slat[22] -&gt; beam_wrap_top</t>
+          <t>beam_wrap_face -&gt; beam</t>
         </is>
       </c>
       <c r="B70" s="2" t="n">
@@ -7602,19 +7602,19 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>1 x #8 x 3, OFFSET INBOARD. slat[22] runs x 105.5 to 107 and the LVL ends at 106.25, so only 3/4 of its 1-1/2 width has beam under the cap - the rest is over beam_end_cap, 3/4 ply. A centred screw lands half in ply. Found by the kernel ray cast.</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. in two rows into the LVL - 3/4 of ply then 1-1/4 into 1-3/4 of beam. Rev AT: OVER x 0 TO 27 THIS IS STRUCTURAL, not a finish fixing: tighten to 6 in o.c. in two rows and glue the full contact area. This panel is the notch reinforcement (see beam_tongue) - it straddles the re-entrant corner at x 3, z 57.25 and runs the full length past the shoulder, so it carries across the corner in shear what the LVL would otherwise carry in cross-grain tension. Keep every screw at least 1 in clear of the corner and out of the notch void below z 57.25 at x 0-3. Rev AT: the wrap had no connection row at all before this - its fixing was never specified and never checked.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>ledge_cleat -&gt; wall:bed</t>
+          <t>beam_wrap_face -&gt; beam_tongue</t>
         </is>
       </c>
       <c r="B71" s="3" t="n">
@@ -7622,23 +7622,23 @@
       </c>
       <c r="C71" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D71" s="3" t="inlineStr">
         <is>
-          <t>2 x 3 in screws into every stud — it carries half an 8 wide lid and whatever is set on it, so it is fixed like a ledger, not tacked like trim</t>
+          <t>glue only over x 0 to 3 - no screws within 1 in of the notch corner at x 3, z 57.25, which is what the beam row already says. Rev AY: this row exists so the arithmetic covers the whole board. beam_tongue is part_of beam - the SAME LVL - but resolve() does not merge part_of members, so beam_wrap_face -&gt; beam checked only 103 1/4 of the 106 1/4 and the 3 the splice exists to protect sat outside every overlap number reported. Found by connection-checker at Rev AX. No physical change: the wood is continuous across x 3 above z 57.25, and the tongue has its own verified gravity path onto side_ledger and deck_joist_tail.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>ledge_strut[*] -&gt; ledge_cleat</t>
+          <t>beam_wrap_face -&gt; side_ledger</t>
         </is>
       </c>
       <c r="B72" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
@@ -7647,18 +7647,18 @@
       </c>
       <c r="D72" s="2" t="inlineStr">
         <is>
-          <t>2 x #8 x 2-1/2 toe-driven into the cleat, plus adhesive</t>
+          <t>#8 x 2-1/2 at 6 in o.c. into the ledger's y-50 end face, over z 53.75-57.25. Rev AT: part of the notch splice - this is what ties the tongue back to the member it bears on. End-grain withdrawal is poor and irrelevant here: the joint works in shear. Rev AY: 2-1/2 not 2, for 1-3/4 of embedment instead of 1-1/4. This is the anchor side of the whole splice claim and 1-1/4 of dowel action in end grain was thin.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>ledge_strut[*] -&gt; ledge_front_rail</t>
+          <t>beam_wrap_face -&gt; deck_joist_tail</t>
         </is>
       </c>
       <c r="B73" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C73" s="3" t="inlineStr">
         <is>
@@ -7667,34 +7667,34 @@
       </c>
       <c r="D73" s="3" t="inlineStr">
         <is>
-          <t>adhesive + 2 pocket screws from inside the well, angled out of the strut into the back of the rail. Pocket, not toe: a toe screw into 3/4 of poplar from behind breaks out the face, and a screw through the rail's face lands in the strut's end grain.</t>
+          <t>#8 x 2-1/2 at 6 in o.c. into the tail's y-50 end face, over z 53.75-57.25 - the other half of the notch splice, into the joist sistered to the ledger (Rev AT; 2-1/2 since Rev AY, same end-grain reason as the ledger half)</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_strut[*]</t>
+          <t>beam_wrap_inner -&gt; beam</t>
         </is>
       </c>
       <c r="B74" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4, 2 per strut, countersunk and filled</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL. Rev AT: finish fixing only - this panel starts at z 58, 3/4 above the notch corner, so it does no structural work and is not part of the splice. It had no connection row either.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_cleat</t>
+          <t>beam_wrap_top -&gt; beam</t>
         </is>
       </c>
       <c r="B75" s="3" t="n">
@@ -7707,34 +7707,34 @@
       </c>
       <c r="D75" s="3" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4 at 12 in o.c., countersunk and filled — the lid is fixed, not hinged</t>
+          <t>construction adhesive + #8 x 2 at 12 in o.c. into the LVL, between the slats. The cap is finish stock doing structural work - it is the slats' seat - so it is fixed on its own account, not by the slat screws alone.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>ledge_cleat_rail -&gt; ledge_front_rail</t>
+          <t>slat[*] -&gt; beam_wrap_top</t>
         </is>
       </c>
       <c r="B76" s="2" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-1/4 at 12 in o.c. from inside the well, through the cleat into the rail — screwed from the back so nothing shows on the face</t>
+          <t>1 x #8 x 3 through the cap into the LVL — 3/4 of cap, 2-1/4 into the beam. Rev AG settles what Rev T left open. slat[22] is the one exception - see below.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>ledge_cleat_rail -&gt; deck_ply</t>
+          <t>slat[22] -&gt; beam_wrap_top</t>
         </is>
       </c>
       <c r="B77" s="3" t="n">
@@ -7747,14 +7747,14 @@
       </c>
       <c r="D77" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #10 x 3-1/2 down through the cleat and the ply into a joist at each of the 9 joists, and #8 x 2 into the ply between them</t>
+          <t>1 x #8 x 3, OFFSET INBOARD. slat[22] runs x 105.5 to 107 and the LVL ends at 106.25, so only 3/4 of its 1-1/2 width has beam under the cap - the rest is over beam_end_cap, 3/4 ply. A centred screw lands half in ply. Found by the kernel ray cast.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_front_rail</t>
+          <t>ledge_cleat -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B78" s="2" t="n">
@@ -7762,23 +7762,23 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4 at 12 in o.c. into the rail's 3/4 top edge, countersunk and filled. Rev AM: the lid is fixed, never hinged, so this joint is permanent - and with the three struts holding the rail's top on 7.25 it is a flush line the whole 106 1/4, not a joint that has to be pulled closed at assembly.</t>
+          <t>2 x 3 in screws into every stud — it carries half an 8 wide lid and whatever is set on it, so it is fixed like a ledger, not tacked like trim</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>ledge_rail_splice -&gt; ledge_front_rail</t>
+          <t>ledge_strut[*] -&gt; ledge_cleat</t>
         </is>
       </c>
       <c r="B79" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C79" s="3" t="inlineStr">
         <is>
@@ -7787,38 +7787,38 @@
       </c>
       <c r="D79" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + #8 x 1-1/4 at 6 in o.c. in two rows, from inside the well through the splice into the back of both rail pieces - 1/2 into the rail's 3/4</t>
+          <t>2 x #8 x 2-1/2 toe-driven into the cleat, plus adhesive</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>ledge_lid -&gt; ledge_end_cap</t>
+          <t>ledge_strut[*] -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B80" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>bearing</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
         <is>
-          <t>#8 x 1-1/4, 2 off — the 3/4 x 8 of skirt top edge the lid laps at the stair end (Rev AH)</t>
+          <t>adhesive + 2 pocket screws from inside the well, angled out of the strut into the back of the rail. Pocket, not toe: a toe screw into 3/4 of poplar from behind breaks out the face, and a screw through the rail's face lands in the strut's end grain.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>screen_top_plate -&gt; slat[*]</t>
+          <t>ledge_lid -&gt; ledge_strut[*]</t>
         </is>
       </c>
       <c r="B81" s="3" t="n">
-        <v>23</v>
+        <v>3</v>
       </c>
       <c r="C81" s="3" t="inlineStr">
         <is>
@@ -7827,14 +7827,14 @@
       </c>
       <c r="D81" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + 1 x #8 x 2-1/2 angled up through the slat into the plate, driven from the loft side, countersunk and filled; 2 x 1-1/2 16ga pins each slat to hold it while the adhesive cures. Rev AS: was UNSPECIFIED. 16ga alone was proposed and is not enough - the structure table calls this screen the GUARD for a 58 deck, and the ceiling note says a 200 lb lean at its top overloads the slat bases. One real screw per slat at each end (the base already has #8 x 3 into the LVL) makes the top a positive connection; the pins are for assembly, not for load.</t>
+          <t>#8 x 1-1/4, 2 per strut, countersunk and filled</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>screen_top_plate -&gt; ceiling</t>
+          <t>ledge_lid -&gt; ledge_cleat</t>
         </is>
       </c>
       <c r="B82" s="2" t="n">
@@ -7842,19 +7842,19 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>ceiling</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
         <is>
-          <t>into ceiling framing / blocking — joist location not yet measured</t>
+          <t>#8 x 1-1/4 at 12 in o.c., countersunk and filled — the lid is fixed, not hinged</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>lnd_ledger_bedwall -&gt; wall:bed</t>
+          <t>ledge_cleat_rail -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B83" s="3" t="n">
@@ -7862,19 +7862,19 @@
       </c>
       <c r="C83" s="3" t="inlineStr">
         <is>
-          <t>wall</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D83" s="3" t="inlineStr">
         <is>
-          <t>3/8 x 4 lags, 2 per stud</t>
+          <t>construction adhesive + #8 x 1-1/4 at 12 in o.c. from inside the well, through the cleat into the rail — screwed from the back so nothing shows on the face</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>stringer_b -&gt; lnd_rim</t>
+          <t>ledge_cleat_rail -&gt; deck_ply</t>
         </is>
       </c>
       <c r="B84" s="2" t="n">
@@ -7882,19 +7882,19 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>3 x 1/4 x 3-1/2 SDS from inside the box through the rim, before the deck goes on</t>
+          <t>construction adhesive + #10 x 3-1/2 down through the cleat and the ply into a joist at each of the 9 joists, and #8 x 2 into the ply between them</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>stringer_c -&gt; lnd_ledger_rightwall</t>
+          <t>ledge_lid -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B85" s="3" t="n">
@@ -7902,19 +7902,19 @@
       </c>
       <c r="C85" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D85" s="3" t="inlineStr">
         <is>
-          <t>plumb cut on the ledger end + 4 x 1/4 x 4-1/2 SDS into right-wall studs</t>
+          <t>#8 x 1-1/4 at 12 in o.c. into the rail's 3/4 top edge, countersunk and filled. Rev AM: the lid is fixed, never hinged, so this joint is permanent - and with the three struts holding the rail's top on 7.25 it is a flush line the whole 106 1/4, not a joint that has to be pulled closed at assembly.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_header</t>
+          <t>ledge_rail_splice -&gt; ledge_front_rail</t>
         </is>
       </c>
       <c r="B86" s="2" t="n">
@@ -7927,14 +7927,14 @@
       </c>
       <c r="D86" s="2" t="inlineStr">
         <is>
-          <t>4 x 1/4 x 3-1/2 SDS over y 18-27. Rev AE: the stringer is on the framing now, not on 3/4 of ply, so a 3-1/2 buries 2 in the header.</t>
+          <t>construction adhesive + #8 x 1-1/4 at 6 in o.c. in two rows, from inside the well through the splice into the back of both rail pieces - 1/2 into the rail's 3/4</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_king_b</t>
+          <t>ledge_lid -&gt; ledge_end_cap</t>
         </is>
       </c>
       <c r="B87" s="3" t="n">
@@ -7942,39 +7942,39 @@
       </c>
       <c r="C87" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D87" s="3" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS</t>
+          <t>#8 x 1-1/4, 2 off — the 3/4 x 8 of skirt top edge the lid laps at the stair end (Rev AH)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; hw_trimmer_b</t>
+          <t>screen_top_plate -&gt; slat[*]</t>
         </is>
       </c>
       <c r="B88" s="2" t="n">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>bearing</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS. Rev AE: the stringer crosses the far jamb pack over z 12-24, so it catches the trimmer as well as the king.</t>
+          <t>construction adhesive + 1 x #8 x 2-1/2 angled up through the slat into the plate, driven from the loft side, countersunk and filled; 2 x 1-1/2 16ga pins each slat to hold it while the adhesive cures. Rev AS: was UNSPECIFIED. 16ga alone was proposed and is not enough - the structure table calls this screen the GUARD for a 58 deck, and the ceiling note says a 200 lb lean at its top overloads the slat bases. One real screw per slat at each end (the base already has #8 x 3 into the LVL) makes the top a positive connection; the pins are for assembly, not for load.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>hw_rake_nailer -&gt; stringer_a</t>
+          <t>screen_top_plate -&gt; ceiling</t>
         </is>
       </c>
       <c r="B89" s="3" t="n">
@@ -7982,19 +7982,19 @@
       </c>
       <c r="C89" s="3" t="inlineStr">
         <is>
-          <t>face-screw</t>
+          <t>ceiling</t>
         </is>
       </c>
       <c r="D89" s="3" t="inlineStr">
         <is>
-          <t>construction adhesive + 6 x 3 in screws toe-driven through the nailer into the stringer's face. Rev AE: the nailer's raked end (1-1/2 x 30 on the slope) dies straight onto stringer A now that the sheathing between them is gone.</t>
+          <t>into ceiling framing / blocking — joist location not yet measured</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>lnd_rim -&gt; hw_header</t>
+          <t>lnd_ledger_bedwall -&gt; wall:bed</t>
         </is>
       </c>
       <c r="B90" s="2" t="n">
@@ -8002,19 +8002,19 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>wall</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>HUC28 concealed-flange hanger, SD10212 screws straight into the header (flanges would foul the side member on an LUS). Rev AE: no 3/4 facing in the path.</t>
+          <t>3/8 x 4 lags, 2 per stud</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>lnd_rim -&gt; lnd_ledger_rightwall</t>
+          <t>stringer_b -&gt; lnd_rim</t>
         </is>
       </c>
       <c r="B91" s="3" t="n">
@@ -8022,59 +8022,59 @@
       </c>
       <c r="C91" s="3" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D91" s="3" t="inlineStr">
         <is>
-          <t>HUC28 concealed-flange hanger (an LUS flange would hang past the ledger end)</t>
+          <t>3 x 1/4 x 3-1/2 SDS from inside the box through the rim, before the deck goes on</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
         <is>
-          <t>lnd_joist[*] -&gt; lnd_ledger_bedwall</t>
+          <t>stringer_c -&gt; lnd_ledger_rightwall</t>
         </is>
       </c>
       <c r="B92" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
         <is>
-          <t>LUS24</t>
+          <t>plumb cut on the ledger end + 4 x 1/4 x 4-1/2 SDS into right-wall studs</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>lnd_joist[*] -&gt; lnd_rim</t>
+          <t>stringer_a -&gt; hw_header</t>
         </is>
       </c>
       <c r="B93" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C93" s="3" t="inlineStr">
         <is>
-          <t>hanger</t>
+          <t>face-screw</t>
         </is>
       </c>
       <c r="D93" s="3" t="inlineStr">
         <is>
-          <t>LUS24 on the rim's back face</t>
+          <t>4 x 1/4 x 3-1/2 SDS over y 18-27. Rev AE: the stringer is on the framing now, not on 3/4 of ply, so a 3-1/2 buries 2 in the header.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
         <is>
-          <t>lnd_side_member -&gt; lnd_rim</t>
+          <t>stringer_a -&gt; hw_king_b</t>
         </is>
       </c>
       <c r="B94" s="2" t="n">
@@ -8087,14 +8087,14 @@
       </c>
       <c r="D94" s="2" t="inlineStr">
         <is>
-          <t>2 x A35 at the inside corner, installed before the joists</t>
+          <t>2 x 1/4 x 3-1/2 SDS</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>stringer_a -&gt; lnd_rim</t>
+          <t>stringer_a -&gt; hw_trimmer_b</t>
         </is>
       </c>
       <c r="B95" s="3" t="n">
@@ -8107,32 +8107,172 @@
       </c>
       <c r="D95" s="3" t="inlineStr">
         <is>
-          <t>2 x 1/4 x 3-1/2 SDS toe-screwed from the stringer's outer face; the side member blocks access from inside the box</t>
+          <t>2 x 1/4 x 3-1/2 SDS. Rev AE: the stringer crosses the far jamb pack over z 12-24, so it catches the trimmer as well as the king.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
         <is>
+          <t>hw_rake_nailer -&gt; stringer_a</t>
+        </is>
+      </c>
+      <c r="B96" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C96" s="2" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>construction adhesive + 6 x 3 in screws toe-driven through the nailer into the stringer's face. Rev AE: the nailer's raked end (1-1/2 x 30 on the slope) dies straight onto stringer A now that the sheathing between them is gone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
+        <is>
+          <t>lnd_rim -&gt; hw_header</t>
+        </is>
+      </c>
+      <c r="B97" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C97" s="3" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D97" s="3" t="inlineStr">
+        <is>
+          <t>HUC28 concealed-flange hanger, SD10212 screws straight into the header (flanges would foul the side member on an LUS). Rev AE: no 3/4 facing in the path.</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>lnd_rim -&gt; lnd_ledger_rightwall</t>
+        </is>
+      </c>
+      <c r="B98" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C98" s="2" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>HUC28 concealed-flange hanger (an LUS flange would hang past the ledger end)</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="3" t="inlineStr">
+        <is>
+          <t>lnd_joist[*] -&gt; lnd_ledger_bedwall</t>
+        </is>
+      </c>
+      <c r="B99" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C99" s="3" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D99" s="3" t="inlineStr">
+        <is>
+          <t>LUS24</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>lnd_joist[*] -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="C100" s="2" t="inlineStr">
+        <is>
+          <t>hanger</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>LUS24 on the rim's back face</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>lnd_side_member -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B101" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C101" s="3" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D101" s="3" t="inlineStr">
+        <is>
+          <t>2 x A35 at the inside corner, installed before the joists</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>stringer_a -&gt; lnd_rim</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="2" t="inlineStr">
+        <is>
+          <t>face-screw</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>2 x 1/4 x 3-1/2 SDS toe-screwed from the stringer's outer face; the side member blocks access from inside the box</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
+        <is>
           <t>lnd_blocking[*] -&gt; stringer_b</t>
         </is>
       </c>
-      <c r="B96" s="2" t="n">
+      <c r="B103" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C96" s="2" t="inlineStr">
+      <c r="C103" s="3" t="inlineStr">
         <is>
           <t>face-screw</t>
         </is>
       </c>
-      <c r="D96" s="2" t="inlineStr">
+      <c r="D103" s="3" t="inlineStr">
         <is>
           <t>2 x 3 in screws each end, toe-driven</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D96"/>
+  <autoFilter ref="A1:D103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -8176,7 +8316,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Generated from dimensions.yaml rev AX</t>
+          <t>Generated from dimensions.yaml rev AY</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -8215,7 +8355,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>It decides the deck's grade, which is why it matters here. The mattress covers y 8 3/4 to 46 3/4 out to about x 77; the rest is walked on and nothing in the model covers it. If it is the finished floor it wants a sanded, paintable face and sealed edges rather than rated sheathing — and the whole 3 sheets move to the paint-grade group. Nesting is indifferent: 3/4 ply comes to the same 10 sheets whether it is bought as one pool or split by grade, so this is purely about the product and the price, not the quantity.</t>
+          <t>The mattress covers y 8 3/4 to 46 3/4 out to about x 77; the rest is walked on and nothing in the model covers it, so the deck is the finished floor and takes a sanded paintable face rather than rated sheathing. Consequence: there is no hidden 3/4 ply left in the build, so the two grade groups collapsed to ONE paint-grade pool — and the sheet count assumes that. Buying the deck as sheathing again would break the nest, not just change the price.</t>
         </is>
       </c>
     </row>
@@ -8232,7 +8372,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Pending price and availability. Three ply grades are needed and they are not interchangeable: structural (deck_ply, the half-wall sheathing), paint-grade show faces (beam wrap, ledge rail and lid, treads, risers, nook lining), and 1/2 flitches (jamb packs, the header's middle ply).</t>
+          <t>Pending price and availability. TWO ply grades, not three: one 3/4 paint-grade pool covering every 3/4 piece including the deck, and 1/2 flitches for the jamb packs and the header's middle ply. Framing species/grade and the slat stock are also open.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update sheet note re kerf and factory edge; remove dead function
</commit_message>
<xml_diff>
--- a/materials/materials-list.xlsx
+++ b/materials/materials-list.xlsx
@@ -8573,12 +8573,12 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Sheet counts are shelf-packed, not nested</t>
+          <t>Sheet counts are a real nest, with kerf</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>The Sheet goods tab lists every panel with its real size. Buy the counts as a floor, not a ceiling, and lay out the deck and the loft ceiling on paper first: both are OVER 48 in y (48 1/4 and 50), so that dimension has to run along the sheet's 8 ft length and each takes one sheet per piece.</t>
+          <t>Every piece is placed by a guillotine first-fit-decreasing nest that reserves 1/8 on every cut, so the Cut layout tab and materials/cut-layout.svg are a layout you can mark out, not an indicative count — the diagrams draw each piece at its finished size with the kerf as the gap between them, and no two pieces overlap or run off a sheet (asserted at build time). Rotation is allowed and the layout flags which pieces came out turned, so an appearance call can override one. TWO CAVEATS. There is no factory-edge trim allowance: the first piece sits in the corner, so the layout assumes two usable edges — kerf IS reserved against the far edge, which is roughly the 1/8 back. And the deck and the loft ceiling are OVER 48 in y (48 1/4 and 50), so that dimension has to run along the sheet's 8 ft length and each takes one sheet per piece.</t>
         </is>
       </c>
     </row>

</xml_diff>